<commit_message>
Lista de precios: tomada del CRM en vez de Shopify
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015XoTitFW4NKs6Tkz8h27S9
</commit_message>
<xml_diff>
--- a/docs/meta-ia/lista-precios-martinez-motos.xlsx
+++ b/docs/meta-ia/lista-precios-martinez-motos.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lista de precios" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Lista de precios'!$A$5:$H$64</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Lista de precios'!$A$5:$H$72</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Lista de precios'!$5:$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H64"/>
+  <dimension ref="A1:H72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -503,7 +503,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Precios en pesos uruguayos. Fuente: tienda Shopify (martinezmotos.com), 20/10/2026.</t>
+          <t>Precios en pesos uruguayos. Fuente: CRM Martinez Motos (productos activos), 20/10/2026.</t>
         </is>
       </c>
     </row>
@@ -527,7 +527,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Variante</t>
+          <t>Tipo</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -569,7 +569,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Tipo alerón</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -606,7 +606,7 @@
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>Espejos Finos</t>
+          <t>Tipo alerón</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
@@ -643,7 +643,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Tipo alerón</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -652,7 +652,7 @@
         </is>
       </c>
       <c r="E8" s="5" t="n">
-        <v>2290</v>
+        <v>2390</v>
       </c>
       <c r="F8" s="6">
         <f>ROUND(E8*0.9,0)</f>
@@ -680,7 +680,7 @@
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>Negro</t>
+          <t>De puño</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
@@ -712,12 +712,12 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Espejos Retrovisores De Manubrio Para Moto 22 Mm</t>
+          <t>Espejos de Puño Circulares Moto Universal Manillar 7/8 Negro</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>De puño</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -744,26 +744,26 @@
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>Soportes de celular</t>
+          <t>Espejos</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>Soporte Celular Moto Universal Manillar Negro Ajustable</t>
+          <t>Extensor Espejo Moto Rosca 8mm Int/Ext Horario Universal</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Extensores</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>SOP-CEL-MAN-001</t>
+          <t>EXT-ESP-8F-8F-001</t>
         </is>
       </c>
       <c r="E11" s="9" t="n">
-        <v>490</v>
+        <v>100</v>
       </c>
       <c r="F11" s="10">
         <f>ROUND(E11*0.9,0)</f>
@@ -775,32 +775,32 @@
         </is>
       </c>
       <c r="H11" s="8" t="n">
-        <v>87</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Soportes de celular</t>
+          <t>Espejos</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Soporte Celular Moto Universal Espejo Negro Ajustable</t>
+          <t>Extensor Espejo Moto Rosca 8mm Int/Ext Antihorario Univ</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Extensores</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>SOP-CEL-ESP-001</t>
+          <t>EXT-ESP-8R-8R-001</t>
         </is>
       </c>
       <c r="E12" s="5" t="n">
-        <v>490</v>
+        <v>100</v>
       </c>
       <c r="F12" s="6">
         <f>ROUND(E12*0.9,0)</f>
@@ -812,32 +812,32 @@
         </is>
       </c>
       <c r="H12" s="4" t="n">
-        <v>89</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>Puños</t>
+          <t>Espejos</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Puños Domino Para Moto Manubrio Goma Antideslizante</t>
+          <t>Extensor Espejo Moto Rosca 8mm Int Hor / Ext Antihor</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>Negro</t>
+          <t>Extensores</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>DOM00</t>
+          <t>EXT-ESP-8F-8R-001</t>
         </is>
       </c>
       <c r="E13" s="9" t="n">
-        <v>450</v>
+        <v>100</v>
       </c>
       <c r="F13" s="10">
         <f>ROUND(E13*0.9,0)</f>
@@ -849,32 +849,32 @@
         </is>
       </c>
       <c r="H13" s="8" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Puños</t>
+          <t>Espejos</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Puños Domino Para Moto Manubrio Goma Antideslizante</t>
+          <t>Extensor Espejo Moto Rosca 8mm Int Antihor / Ext Hor</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Rojo</t>
+          <t>Extensores</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>DOM01</t>
+          <t>EXT-ESP-8R-8F-001</t>
         </is>
       </c>
       <c r="E14" s="5" t="n">
-        <v>450</v>
+        <v>100</v>
       </c>
       <c r="F14" s="6">
         <f>ROUND(E14*0.9,0)</f>
@@ -886,32 +886,32 @@
         </is>
       </c>
       <c r="H14" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>Puños</t>
+          <t>Espejos</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>Puños Domino Para Moto Manubrio Goma Antideslizante</t>
+          <t>Extensor Espejo Moto Rosca 8mm Int Hor / 10mm Ext Hor</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>Azul</t>
+          <t>Extensores</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>DOM02</t>
+          <t>EXT-ESP-8F-10F-001</t>
         </is>
       </c>
       <c r="E15" s="9" t="n">
-        <v>450</v>
+        <v>100</v>
       </c>
       <c r="F15" s="10">
         <f>ROUND(E15*0.9,0)</f>
@@ -923,32 +923,32 @@
         </is>
       </c>
       <c r="H15" s="8" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Puños</t>
+          <t>Espejos</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Puños Domino Para Moto Manubrio Goma Antideslizante</t>
+          <t>Extensor Espejo Moto Rosca 8mm Int Hor / 10mm Ext Antihor</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Naranja</t>
+          <t>Extensores</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>DOM03</t>
+          <t>EXT-ESP-8F-10R-001</t>
         </is>
       </c>
       <c r="E16" s="5" t="n">
-        <v>450</v>
+        <v>100</v>
       </c>
       <c r="F16" s="6">
         <f>ROUND(E16*0.9,0)</f>
@@ -960,32 +960,32 @@
         </is>
       </c>
       <c r="H16" s="4" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>Puños</t>
+          <t>Espejos</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>Puños Domino Para Moto Manubrio Goma Antideslizante</t>
+          <t>Extensor Espejo Moto Rosca 8mm Int Antihor / 10mm Ext</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>Verde</t>
+          <t>Extensores</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>DOM04</t>
+          <t>EXT-ESP-8R-10F-001</t>
         </is>
       </c>
       <c r="E17" s="9" t="n">
-        <v>450</v>
+        <v>100</v>
       </c>
       <c r="F17" s="10">
         <f>ROUND(E17*0.9,0)</f>
@@ -997,32 +997,32 @@
         </is>
       </c>
       <c r="H17" s="8" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Puños</t>
+          <t>Espejos</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Puños Universales Antideslizantes Con Contrapesos Anticaídas</t>
+          <t>Extensor Espejo Moto Rosca 8mm Int/10mm Ext Antihorario</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Negro</t>
+          <t>Extensores</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>PUNBLACK</t>
+          <t>EXT-ESP-8R-10R-001</t>
         </is>
       </c>
       <c r="E18" s="5" t="n">
-        <v>990</v>
+        <v>100</v>
       </c>
       <c r="F18" s="6">
         <f>ROUND(E18*0.9,0)</f>
@@ -1034,32 +1034,32 @@
         </is>
       </c>
       <c r="H18" s="4" t="n">
-        <v>21</v>
+        <v>10</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>Puños</t>
+          <t>Espejos</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>Puños Universales Antideslizantes Con Contrapesos Anticaídas</t>
+          <t>Extensor Espejo Moto Rosca 10mm Int/Ext Horario Universal</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>Dorado</t>
+          <t>Extensores</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>PUNYELLOW</t>
+          <t>EXT-ESP-10F-10F-001</t>
         </is>
       </c>
       <c r="E19" s="9" t="n">
-        <v>990</v>
+        <v>100</v>
       </c>
       <c r="F19" s="10">
         <f>ROUND(E19*0.9,0)</f>
@@ -1071,106 +1071,106 @@
         </is>
       </c>
       <c r="H19" s="8" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="12" t="inlineStr">
-        <is>
-          <t>Puños</t>
-        </is>
-      </c>
-      <c r="B20" s="12" t="inlineStr">
-        <is>
-          <t>Puños Universales Antideslizantes Con Contrapesos Anticaídas</t>
-        </is>
-      </c>
-      <c r="C20" s="12" t="inlineStr">
-        <is>
-          <t>Rojo</t>
-        </is>
-      </c>
-      <c r="D20" s="12" t="inlineStr">
-        <is>
-          <t>PUNRED</t>
-        </is>
-      </c>
-      <c r="E20" s="13" t="n">
-        <v>990</v>
-      </c>
-      <c r="F20" s="14">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Espejos</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Extensor Espejo Moto Rosca 10mm Int/Ext Antihorario Univ</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Extensores</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>EXT-ESP-10R-10R-001</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F20" s="6">
         <f>ROUND(E20*0.9,0)</f>
         <v/>
       </c>
-      <c r="G20" s="12" t="inlineStr">
-        <is>
-          <t>Sin stock</t>
-        </is>
-      </c>
-      <c r="H20" s="12" t="n">
-        <v>0</v>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>Con stock</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="15" t="inlineStr">
-        <is>
-          <t>Puños</t>
-        </is>
-      </c>
-      <c r="B21" s="15" t="inlineStr">
-        <is>
-          <t>Puños Universales Antideslizantes Con Contrapesos Anticaídas</t>
-        </is>
-      </c>
-      <c r="C21" s="15" t="inlineStr">
-        <is>
-          <t>Naranja</t>
-        </is>
-      </c>
-      <c r="D21" s="15" t="inlineStr">
-        <is>
-          <t>PUNORGANG</t>
-        </is>
-      </c>
-      <c r="E21" s="16" t="n">
-        <v>990</v>
-      </c>
-      <c r="F21" s="17">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>Espejos</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>Extensor Espejo Moto Rosca 10mm Int Hor / Ext Antihor</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Extensores</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>EXT-ESP-10F-10R-001</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="F21" s="10">
         <f>ROUND(E21*0.9,0)</f>
         <v/>
       </c>
-      <c r="G21" s="15" t="inlineStr">
-        <is>
-          <t>Sin stock</t>
-        </is>
-      </c>
-      <c r="H21" s="15" t="n">
-        <v>0</v>
+      <c r="G21" s="11" t="inlineStr">
+        <is>
+          <t>Con stock</t>
+        </is>
+      </c>
+      <c r="H21" s="8" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>Puños</t>
+          <t>Espejos</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Par De Puños Estilo Metálico Para Motos Chopper Café Racer Plateado</t>
+          <t>Extensor Espejo Moto Rosca 10mm Int Antihor / Ext Hor</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Extensores</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>SBJ-10078</t>
+          <t>EXT-ESP-10R-10F-001</t>
         </is>
       </c>
       <c r="E22" s="5" t="n">
-        <v>1670</v>
+        <v>100</v>
       </c>
       <c r="F22" s="6">
         <f>ROUND(E22*0.9,0)</f>
@@ -1182,32 +1182,32 @@
         </is>
       </c>
       <c r="H22" s="4" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>Manillares</t>
+          <t>Espejos</t>
         </is>
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>Manillar Universal Aluminio Para Moto 22mm</t>
+          <t>Extensor Espejo Moto Rosca 10mm Int Hor / 8mm Ext Hor</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>Negro</t>
+          <t>Extensores</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>HP-CB0381</t>
+          <t>EXT-ESP-10F-8F-001</t>
         </is>
       </c>
       <c r="E23" s="9" t="n">
-        <v>1190</v>
+        <v>100</v>
       </c>
       <c r="F23" s="10">
         <f>ROUND(E23*0.9,0)</f>
@@ -1219,32 +1219,32 @@
         </is>
       </c>
       <c r="H23" s="8" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Manillares</t>
+          <t>Espejos</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Manillar Universal Aluminio Para Moto 22mm</t>
+          <t>Extensor Espejo Moto Rosca 10mm Int Hor / 8mm Ext Antihor</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Blanco</t>
+          <t>Extensores</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>HP-CB0382</t>
+          <t>EXT-ESP-10F-8R-001</t>
         </is>
       </c>
       <c r="E24" s="5" t="n">
-        <v>1190</v>
+        <v>100</v>
       </c>
       <c r="F24" s="6">
         <f>ROUND(E24*0.9,0)</f>
@@ -1256,32 +1256,32 @@
         </is>
       </c>
       <c r="H24" s="4" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>Manillares</t>
+          <t>Espejos</t>
         </is>
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>Manillar Universal Aluminio Para Moto 22mm</t>
+          <t>Extensor Espejo Moto Rosca 10mm Int Antihor / 8mm Ext</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>Amarillo</t>
+          <t>Extensores</t>
         </is>
       </c>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t>HP-CB0383</t>
+          <t>EXT-ESP-10R-8F-001</t>
         </is>
       </c>
       <c r="E25" s="9" t="n">
-        <v>1190</v>
+        <v>100</v>
       </c>
       <c r="F25" s="10">
         <f>ROUND(E25*0.9,0)</f>
@@ -1293,32 +1293,32 @@
         </is>
       </c>
       <c r="H25" s="8" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>Manillares</t>
+          <t>Espejos</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Manillar Universal Aluminio Para Moto 22mm</t>
+          <t>Extensor Espejo Moto Rosca 10mm Int/8mm Ext Antihorario</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Azul</t>
+          <t>Extensores</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>HP-CB0384</t>
+          <t>EXT-ESP-10R-8R-001</t>
         </is>
       </c>
       <c r="E26" s="5" t="n">
-        <v>1190</v>
+        <v>100</v>
       </c>
       <c r="F26" s="6">
         <f>ROUND(E26*0.9,0)</f>
@@ -1330,32 +1330,32 @@
         </is>
       </c>
       <c r="H26" s="4" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>Manillares</t>
+          <t>Soportes y bases</t>
         </is>
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>Manillar Universal Aluminio Para Moto 22mm</t>
+          <t>Soporte Celular Moto Universal Manillar Negro Ajustable</t>
         </is>
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>Rojo</t>
+          <t>Soportes de celular</t>
         </is>
       </c>
       <c r="D27" s="8" t="inlineStr">
         <is>
-          <t>HP-CB0385</t>
+          <t>SOP-CEL-MAN-001</t>
         </is>
       </c>
       <c r="E27" s="9" t="n">
-        <v>1190</v>
+        <v>490</v>
       </c>
       <c r="F27" s="10">
         <f>ROUND(E27*0.9,0)</f>
@@ -1367,32 +1367,32 @@
         </is>
       </c>
       <c r="H27" s="8" t="n">
-        <v>5</v>
+        <v>87</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>Manillares</t>
+          <t>Soportes y bases</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Manillar Para Moto Custom Chopper En Acero Cromado Y Negro</t>
+          <t>Soporte Celular Moto Universal Espejo Negro Ajustable</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Negro</t>
+          <t>Soportes de celular</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>MAN-78-V2-NEG-001</t>
+          <t>SOP-CEL-ESP-001</t>
         </is>
       </c>
       <c r="E28" s="5" t="n">
-        <v>690</v>
+        <v>490</v>
       </c>
       <c r="F28" s="6">
         <f>ROUND(E28*0.9,0)</f>
@@ -1404,32 +1404,32 @@
         </is>
       </c>
       <c r="H28" s="4" t="n">
-        <v>5</v>
+        <v>89</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>Manillares</t>
+          <t>Soportes y bases</t>
         </is>
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>Manillar Para Moto Custom Chopper En Acero Cromado Y Negro</t>
+          <t>Extensor De Pie Pata Lateral Moto Bicicleta Base Soporte Negro</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>Plateado</t>
+          <t>Pata lateral</t>
         </is>
       </c>
       <c r="D29" s="8" t="inlineStr">
         <is>
-          <t>MAN-78-V2-PLA-001</t>
+          <t>YTLY-30</t>
         </is>
       </c>
       <c r="E29" s="9" t="n">
-        <v>690</v>
+        <v>274</v>
       </c>
       <c r="F29" s="10">
         <f>ROUND(E29*0.9,0)</f>
@@ -1441,106 +1441,106 @@
         </is>
       </c>
       <c r="H29" s="8" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>Manillares</t>
-        </is>
-      </c>
-      <c r="B30" s="4" t="inlineStr">
-        <is>
-          <t>Manillar Café Racer Universal 7/8 22mm Recto Negro</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D30" s="4" t="inlineStr">
-        <is>
-          <t>MAN-78-V3-NEG-001</t>
-        </is>
-      </c>
-      <c r="E30" s="5" t="n">
-        <v>890</v>
-      </c>
-      <c r="F30" s="6">
+      <c r="A30" s="12" t="inlineStr">
+        <is>
+          <t>Soportes y bases</t>
+        </is>
+      </c>
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>Gato Soporte Elevador Moto Rueda Trasera Delantera 350kgs - Negro</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="inlineStr">
+        <is>
+          <t>Gatos elevadores</t>
+        </is>
+      </c>
+      <c r="D30" s="12" t="inlineStr">
+        <is>
+          <t>GZTYJ-41046N</t>
+        </is>
+      </c>
+      <c r="E30" s="13" t="n">
+        <v>2890</v>
+      </c>
+      <c r="F30" s="14">
         <f>ROUND(E30*0.9,0)</f>
         <v/>
       </c>
-      <c r="G30" s="7" t="inlineStr">
-        <is>
-          <t>Con stock</t>
-        </is>
-      </c>
-      <c r="H30" s="4" t="n">
-        <v>2</v>
+      <c r="G30" s="12" t="inlineStr">
+        <is>
+          <t>Sin stock</t>
+        </is>
+      </c>
+      <c r="H30" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="8" t="inlineStr">
-        <is>
-          <t>Manillares</t>
-        </is>
-      </c>
-      <c r="B31" s="8" t="inlineStr">
-        <is>
-          <t>Anti Shimmy Manillar Universal Moto Aluminio Negro</t>
-        </is>
-      </c>
-      <c r="C31" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D31" s="8" t="inlineStr">
-        <is>
-          <t>HP-MG072</t>
-        </is>
-      </c>
-      <c r="E31" s="9" t="n">
-        <v>990</v>
-      </c>
-      <c r="F31" s="10">
+      <c r="A31" s="15" t="inlineStr">
+        <is>
+          <t>Soportes y bases</t>
+        </is>
+      </c>
+      <c r="B31" s="15" t="inlineStr">
+        <is>
+          <t>Gato Soporte Elevador Moto Rueda Trasera Delantera 350kgs - Rojo</t>
+        </is>
+      </c>
+      <c r="C31" s="15" t="inlineStr">
+        <is>
+          <t>Gatos elevadores</t>
+        </is>
+      </c>
+      <c r="D31" s="15" t="inlineStr">
+        <is>
+          <t>GZTYJ-41046R</t>
+        </is>
+      </c>
+      <c r="E31" s="16" t="n">
+        <v>2890</v>
+      </c>
+      <c r="F31" s="17">
         <f>ROUND(E31*0.9,0)</f>
         <v/>
       </c>
-      <c r="G31" s="11" t="inlineStr">
-        <is>
-          <t>Con stock</t>
-        </is>
-      </c>
-      <c r="H31" s="8" t="n">
-        <v>2</v>
+      <c r="G31" s="15" t="inlineStr">
+        <is>
+          <t>Sin stock</t>
+        </is>
+      </c>
+      <c r="H31" s="15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Puños</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Guardamanos Protector Puños Moto Enduro Cross ABS</t>
+          <t>Puños Domino Para Moto Manubrio Goma Antideslizante Negro</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Negro</t>
+          <t>Domino</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>HP-Q0211</t>
+          <t>DOM00</t>
         </is>
       </c>
       <c r="E32" s="5" t="n">
-        <v>690</v>
+        <v>450</v>
       </c>
       <c r="F32" s="6">
         <f>ROUND(E32*0.9,0)</f>
@@ -1552,32 +1552,32 @@
         </is>
       </c>
       <c r="H32" s="4" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Puños</t>
         </is>
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>Guardamanos Protector Puños Moto Enduro Cross ABS</t>
+          <t>Puños Domino Para Moto Manubrio Goma Antideslizante Rojo</t>
         </is>
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>Azul</t>
+          <t>Domino</t>
         </is>
       </c>
       <c r="D33" s="8" t="inlineStr">
         <is>
-          <t>HP-Q0212</t>
+          <t>DOM01</t>
         </is>
       </c>
       <c r="E33" s="9" t="n">
-        <v>690</v>
+        <v>450</v>
       </c>
       <c r="F33" s="10">
         <f>ROUND(E33*0.9,0)</f>
@@ -1589,32 +1589,32 @@
         </is>
       </c>
       <c r="H33" s="8" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Puños</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Guardamanos Protector Puños Moto Enduro Cross ABS</t>
+          <t>Puños Domino Para Moto Manubrio Goma Antideslizante Azul</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Rojo</t>
+          <t>Domino</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>HP-Q0213</t>
+          <t>DOM02</t>
         </is>
       </c>
       <c r="E34" s="5" t="n">
-        <v>690</v>
+        <v>450</v>
       </c>
       <c r="F34" s="6">
         <f>ROUND(E34*0.9,0)</f>
@@ -1626,32 +1626,32 @@
         </is>
       </c>
       <c r="H34" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Puños</t>
         </is>
       </c>
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>Guardamanos Moto Con Señalero LED Integrado Negro</t>
+          <t>Puños Domino Para Moto Manubrio Goma Antideslizante Naranja</t>
         </is>
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Domino</t>
         </is>
       </c>
       <c r="D35" s="8" t="inlineStr">
         <is>
-          <t>HP-HS010</t>
+          <t>DOM03</t>
         </is>
       </c>
       <c r="E35" s="9" t="n">
-        <v>990</v>
+        <v>450</v>
       </c>
       <c r="F35" s="10">
         <f>ROUND(E35*0.9,0)</f>
@@ -1663,32 +1663,32 @@
         </is>
       </c>
       <c r="H35" s="8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Puños</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Protector De Levas Universal Moto ABS Varios Colores</t>
+          <t>Puños Domino Para Moto Manubrio Goma Antideslizante Verde</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Negro</t>
+          <t>Domino</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>HP-Q035B1</t>
+          <t>DOM04</t>
         </is>
       </c>
       <c r="E36" s="5" t="n">
-        <v>890</v>
+        <v>450</v>
       </c>
       <c r="F36" s="6">
         <f>ROUND(E36*0.9,0)</f>
@@ -1700,32 +1700,32 @@
         </is>
       </c>
       <c r="H36" s="4" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Puños</t>
         </is>
       </c>
       <c r="B37" s="8" t="inlineStr">
         <is>
-          <t>Protector De Levas Universal Moto ABS Varios Colores</t>
+          <t>Puños Universales Antideslizantes Con Contrapesos Anticaídas Negro</t>
         </is>
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t>Azul</t>
+          <t>Con contrapeso</t>
         </is>
       </c>
       <c r="D37" s="8" t="inlineStr">
         <is>
-          <t>HP-Q035B2</t>
+          <t>PUNBLACK</t>
         </is>
       </c>
       <c r="E37" s="9" t="n">
-        <v>890</v>
+        <v>990</v>
       </c>
       <c r="F37" s="10">
         <f>ROUND(E37*0.9,0)</f>
@@ -1737,143 +1737,143 @@
         </is>
       </c>
       <c r="H37" s="8" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="12" t="inlineStr">
-        <is>
-          <t>Protección</t>
-        </is>
-      </c>
-      <c r="B38" s="12" t="inlineStr">
-        <is>
-          <t>Protector De Levas Universal Moto ABS Varios Colores</t>
-        </is>
-      </c>
-      <c r="C38" s="12" t="inlineStr">
-        <is>
-          <t>Rojo</t>
-        </is>
-      </c>
-      <c r="D38" s="12" t="inlineStr">
-        <is>
-          <t>HP-Q035B3</t>
-        </is>
-      </c>
-      <c r="E38" s="13" t="n">
-        <v>890</v>
-      </c>
-      <c r="F38" s="14">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Puños</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Puños Universales Antideslizantes Con Contrapesos Anticaídas Dorado</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>Con contrapeso</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>PUNYELLOW</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="n">
+        <v>990</v>
+      </c>
+      <c r="F38" s="6">
         <f>ROUND(E38*0.9,0)</f>
         <v/>
       </c>
-      <c r="G38" s="12" t="inlineStr">
+      <c r="G38" s="7" t="inlineStr">
+        <is>
+          <t>Con stock</t>
+        </is>
+      </c>
+      <c r="H38" s="4" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="15" t="inlineStr">
+        <is>
+          <t>Puños</t>
+        </is>
+      </c>
+      <c r="B39" s="15" t="inlineStr">
+        <is>
+          <t>Puños Universales Antideslizantes Con Contrapesos Anticaídas Rojo</t>
+        </is>
+      </c>
+      <c r="C39" s="15" t="inlineStr">
+        <is>
+          <t>Con contrapeso</t>
+        </is>
+      </c>
+      <c r="D39" s="15" t="inlineStr">
+        <is>
+          <t>PUNRED</t>
+        </is>
+      </c>
+      <c r="E39" s="16" t="n">
+        <v>990</v>
+      </c>
+      <c r="F39" s="17">
+        <f>ROUND(E39*0.9,0)</f>
+        <v/>
+      </c>
+      <c r="G39" s="15" t="inlineStr">
         <is>
           <t>Sin stock</t>
         </is>
       </c>
-      <c r="H38" s="12" t="n">
+      <c r="H39" s="15" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="8" t="inlineStr">
-        <is>
-          <t>Protección</t>
-        </is>
-      </c>
-      <c r="B39" s="8" t="inlineStr">
-        <is>
-          <t>Protector De Levas Freno Y Embrague Estilo Fibra De Carbono Negro</t>
-        </is>
-      </c>
-      <c r="C39" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D39" s="8" t="inlineStr">
-        <is>
-          <t>HS-30006</t>
-        </is>
-      </c>
-      <c r="E39" s="9" t="n">
-        <v>690</v>
-      </c>
-      <c r="F39" s="10">
-        <f>ROUND(E39*0.9,0)</f>
-        <v/>
-      </c>
-      <c r="G39" s="11" t="inlineStr">
-        <is>
-          <t>Con stock</t>
-        </is>
-      </c>
-      <c r="H39" s="8" t="n">
-        <v>20</v>
-      </c>
-    </row>
     <row r="40">
-      <c r="A40" s="4" t="inlineStr">
-        <is>
-          <t>Protección</t>
-        </is>
-      </c>
-      <c r="B40" s="4" t="inlineStr">
-        <is>
-          <t>Slider Universal Aluminio Grande Moto Protector Anti Caídas</t>
-        </is>
-      </c>
-      <c r="C40" s="4" t="inlineStr">
-        <is>
-          <t>Negro</t>
-        </is>
-      </c>
-      <c r="D40" s="4" t="inlineStr">
-        <is>
-          <t>FSB-002</t>
-        </is>
-      </c>
-      <c r="E40" s="5" t="n">
-        <v>1290</v>
-      </c>
-      <c r="F40" s="6">
+      <c r="A40" s="12" t="inlineStr">
+        <is>
+          <t>Puños</t>
+        </is>
+      </c>
+      <c r="B40" s="12" t="inlineStr">
+        <is>
+          <t>Puños Universales Antideslizantes Con Contrapesos Anticaídas Naranja</t>
+        </is>
+      </c>
+      <c r="C40" s="12" t="inlineStr">
+        <is>
+          <t>Con contrapeso</t>
+        </is>
+      </c>
+      <c r="D40" s="12" t="inlineStr">
+        <is>
+          <t>PUNORGANG</t>
+        </is>
+      </c>
+      <c r="E40" s="13" t="n">
+        <v>990</v>
+      </c>
+      <c r="F40" s="14">
         <f>ROUND(E40*0.9,0)</f>
         <v/>
       </c>
-      <c r="G40" s="7" t="inlineStr">
-        <is>
-          <t>Con stock</t>
-        </is>
-      </c>
-      <c r="H40" s="4" t="n">
-        <v>5</v>
+      <c r="G40" s="12" t="inlineStr">
+        <is>
+          <t>Sin stock</t>
+        </is>
+      </c>
+      <c r="H40" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Manillares</t>
         </is>
       </c>
       <c r="B41" s="8" t="inlineStr">
         <is>
-          <t>Slider Universal Aluminio Grande Moto Protector Anti Caídas</t>
+          <t>Manillar Universal Aluminio Para Moto 22mm - Negro</t>
         </is>
       </c>
       <c r="C41" s="8" t="inlineStr">
         <is>
-          <t>Naranja</t>
+          <t>Universal 7/8</t>
         </is>
       </c>
       <c r="D41" s="8" t="inlineStr">
         <is>
-          <t>FSB-003</t>
+          <t>HP-CB0381</t>
         </is>
       </c>
       <c r="E41" s="9" t="n">
-        <v>1290</v>
+        <v>1190</v>
       </c>
       <c r="F41" s="10">
         <f>ROUND(E41*0.9,0)</f>
@@ -1885,32 +1885,32 @@
         </is>
       </c>
       <c r="H41" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>Matrícula</t>
+          <t>Manillares</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>Porta Matricula Rebatible Placa Patente Moto Rebatible</t>
+          <t>Manillar Universal Aluminio Para Moto 22mm - Blanco</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Universal 7/8</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>CPJ-62001</t>
+          <t>HP-CB0382</t>
         </is>
       </c>
       <c r="E42" s="5" t="n">
-        <v>1290</v>
+        <v>1190</v>
       </c>
       <c r="F42" s="6">
         <f>ROUND(E42*0.9,0)</f>
@@ -1922,32 +1922,32 @@
         </is>
       </c>
       <c r="H42" s="4" t="n">
-        <v>38</v>
+        <v>5</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t>Matrícula</t>
+          <t>Manillares</t>
         </is>
       </c>
       <c r="B43" s="8" t="inlineStr">
         <is>
-          <t>Porta Matricula Moto Rebatible Compacto Perfil Bajo Con Luz</t>
+          <t>Manillar Universal Aluminio Para Moto 22mm - Amarillo</t>
         </is>
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Universal 7/8</t>
         </is>
       </c>
       <c r="D43" s="8" t="inlineStr">
         <is>
-          <t>PATENTE1</t>
+          <t>HP-CB0383</t>
         </is>
       </c>
       <c r="E43" s="9" t="n">
-        <v>890</v>
+        <v>1190</v>
       </c>
       <c r="F43" s="10">
         <f>ROUND(E43*0.9,0)</f>
@@ -1959,32 +1959,32 @@
         </is>
       </c>
       <c r="H43" s="8" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>Carenado y parabrisas</t>
+          <t>Manillares</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>Guardabarros Trasero Universal Moto ABS</t>
+          <t>Manillar Universal Aluminio Para Moto 22mm - Azul</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Universal 7/8</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>HP-DB004-B</t>
+          <t>HP-CB0384</t>
         </is>
       </c>
       <c r="E44" s="5" t="n">
-        <v>1290</v>
+        <v>1190</v>
       </c>
       <c r="F44" s="6">
         <f>ROUND(E44*0.9,0)</f>
@@ -1996,32 +1996,32 @@
         </is>
       </c>
       <c r="H44" s="4" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>Carenado y parabrisas</t>
+          <t>Manillares</t>
         </is>
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>Parabrisas Universal 45cm Para Moto Chopper Custom Cruiser Transparente</t>
+          <t>Manillar Universal Aluminio Para Moto 22mm - Rojo</t>
         </is>
       </c>
       <c r="C45" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Universal 7/8</t>
         </is>
       </c>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>HP-DF028</t>
+          <t>HP-CB0385</t>
         </is>
       </c>
       <c r="E45" s="9" t="n">
-        <v>3190</v>
+        <v>1190</v>
       </c>
       <c r="F45" s="10">
         <f>ROUND(E45*0.9,0)</f>
@@ -2033,69 +2033,69 @@
         </is>
       </c>
       <c r="H45" s="8" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="12" t="inlineStr">
-        <is>
-          <t>Carenado y parabrisas</t>
-        </is>
-      </c>
-      <c r="B46" s="12" t="inlineStr">
-        <is>
-          <t>Deflector Parabrisas Para Moto Universal Transparente</t>
-        </is>
-      </c>
-      <c r="C46" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D46" s="12" t="inlineStr">
-        <is>
-          <t>DFB-002</t>
-        </is>
-      </c>
-      <c r="E46" s="13" t="n">
-        <v>1750</v>
-      </c>
-      <c r="F46" s="14">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Manillares</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>Manillar Moto Universal 7/8 22mm Alto Negro Antideslizante</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>MAN-78-V2-NEG-001</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="n">
+        <v>690</v>
+      </c>
+      <c r="F46" s="6">
         <f>ROUND(E46*0.9,0)</f>
         <v/>
       </c>
-      <c r="G46" s="12" t="inlineStr">
-        <is>
-          <t>Sin stock</t>
-        </is>
-      </c>
-      <c r="H46" s="12" t="n">
-        <v>0</v>
+      <c r="G46" s="7" t="inlineStr">
+        <is>
+          <t>Con stock</t>
+        </is>
+      </c>
+      <c r="H46" s="4" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t>Eléctrico</t>
+          <t>Manillares</t>
         </is>
       </c>
       <c r="B47" s="8" t="inlineStr">
         <is>
-          <t>Señaleros LED Finos Universales 12V Para Moto</t>
+          <t>Manillar Moto Universal 7/8 22mm Alto Plateado Antideslizante</t>
         </is>
       </c>
       <c r="C47" s="8" t="inlineStr">
         <is>
-          <t>Negro</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="D47" s="8" t="inlineStr">
         <is>
-          <t>HP-Z0531</t>
+          <t>MAN-78-V2-PLA-001</t>
         </is>
       </c>
       <c r="E47" s="9" t="n">
-        <v>370</v>
+        <v>690</v>
       </c>
       <c r="F47" s="10">
         <f>ROUND(E47*0.9,0)</f>
@@ -2107,32 +2107,32 @@
         </is>
       </c>
       <c r="H47" s="8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>Eléctrico</t>
+          <t>Manillares</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>Señaleros LED Finos Universales 12V Para Moto</t>
+          <t>Manillar Café Racer Universal 7/8 22mm Recto Negro</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Blanco</t>
+          <t>Café Racer</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>HP-Z0532</t>
+          <t>MAN-78-V3-NEG-001</t>
         </is>
       </c>
       <c r="E48" s="5" t="n">
-        <v>370</v>
+        <v>890</v>
       </c>
       <c r="F48" s="6">
         <f>ROUND(E48*0.9,0)</f>
@@ -2144,32 +2144,32 @@
         </is>
       </c>
       <c r="H48" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
         <is>
-          <t>Eléctrico</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="B49" s="8" t="inlineStr">
         <is>
-          <t>Señaleros LED Finos Universales 12V Para Moto</t>
+          <t>Guardamanos Protector Puños Moto Enduro Cross ABS - Negro</t>
         </is>
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>Azul</t>
+          <t>Guardamanos</t>
         </is>
       </c>
       <c r="D49" s="8" t="inlineStr">
         <is>
-          <t>HP-Z0534</t>
+          <t>HP-Q0211</t>
         </is>
       </c>
       <c r="E49" s="9" t="n">
-        <v>370</v>
+        <v>690</v>
       </c>
       <c r="F49" s="10">
         <f>ROUND(E49*0.9,0)</f>
@@ -2181,32 +2181,32 @@
         </is>
       </c>
       <c r="H49" s="8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>Eléctrico</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>Señaleros LED Finos Universales 12V Para Moto</t>
+          <t>Guardamanos Protector Puños Moto Enduro Cross ABS - Azul</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>Rojo</t>
+          <t>Guardamanos</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>HP-Z0535</t>
+          <t>HP-Q0212</t>
         </is>
       </c>
       <c r="E50" s="5" t="n">
-        <v>370</v>
+        <v>690</v>
       </c>
       <c r="F50" s="6">
         <f>ROUND(E50*0.9,0)</f>
@@ -2218,106 +2218,106 @@
         </is>
       </c>
       <c r="H50" s="4" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="inlineStr">
+        <is>
+          <t>Protección</t>
+        </is>
+      </c>
+      <c r="B51" s="8" t="inlineStr">
+        <is>
+          <t>Guardamanos Protector Puños Moto Enduro Cross ABS - Rojo</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>Guardamanos</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>HP-Q0213</t>
+        </is>
+      </c>
+      <c r="E51" s="9" t="n">
+        <v>690</v>
+      </c>
+      <c r="F51" s="10">
+        <f>ROUND(E51*0.9,0)</f>
+        <v/>
+      </c>
+      <c r="G51" s="11" t="inlineStr">
+        <is>
+          <t>Con stock</t>
+        </is>
+      </c>
+      <c r="H51" s="8" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Protección</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>Guardamanos Moto Con Señalero LED Integrado Negro</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>Guardamanos</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>HP-HS010</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="n">
+        <v>990</v>
+      </c>
+      <c r="F52" s="6">
+        <f>ROUND(E52*0.9,0)</f>
+        <v/>
+      </c>
+      <c r="G52" s="7" t="inlineStr">
+        <is>
+          <t>Con stock</t>
+        </is>
+      </c>
+      <c r="H52" s="4" t="n">
         <v>3</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="15" t="inlineStr">
-        <is>
-          <t>Eléctrico</t>
-        </is>
-      </c>
-      <c r="B51" s="15" t="inlineStr">
-        <is>
-          <t>Señaleros LED Finos Universales 12V Para Moto</t>
-        </is>
-      </c>
-      <c r="C51" s="15" t="inlineStr">
-        <is>
-          <t>Amarillo</t>
-        </is>
-      </c>
-      <c r="D51" s="15" t="inlineStr">
-        <is>
-          <t>HP-Z0533</t>
-        </is>
-      </c>
-      <c r="E51" s="16" t="n">
-        <v>370</v>
-      </c>
-      <c r="F51" s="17">
-        <f>ROUND(E51*0.9,0)</f>
-        <v/>
-      </c>
-      <c r="G51" s="15" t="inlineStr">
-        <is>
-          <t>Sin stock</t>
-        </is>
-      </c>
-      <c r="H51" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="12" t="inlineStr">
-        <is>
-          <t>Eléctrico</t>
-        </is>
-      </c>
-      <c r="B52" s="12" t="inlineStr">
-        <is>
-          <t>Señaleros Led Secuenciales Luz Amarilla Universales Moto Amarillo</t>
-        </is>
-      </c>
-      <c r="C52" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D52" s="12" t="inlineStr">
-        <is>
-          <t>SEÑAL01</t>
-        </is>
-      </c>
-      <c r="E52" s="13" t="n">
-        <v>350</v>
-      </c>
-      <c r="F52" s="14">
-        <f>ROUND(E52*0.9,0)</f>
-        <v/>
-      </c>
-      <c r="G52" s="12" t="inlineStr">
-        <is>
-          <t>Sin stock</t>
-        </is>
-      </c>
-      <c r="H52" s="12" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
-          <t>Soportes y bases</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="B53" s="8" t="inlineStr">
         <is>
-          <t>Extensor De Pie Pata Lateral Moto Bicicleta Base Soporte Negro</t>
+          <t>Protector De Levas Universal Moto ABS Varios Colores - Negro</t>
         </is>
       </c>
       <c r="C53" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Protectores de levas</t>
         </is>
       </c>
       <c r="D53" s="8" t="inlineStr">
         <is>
-          <t>YTLY-30</t>
+          <t>HP-Q035B1</t>
         </is>
       </c>
       <c r="E53" s="9" t="n">
-        <v>274</v>
+        <v>890</v>
       </c>
       <c r="F53" s="10">
         <f>ROUND(E53*0.9,0)</f>
@@ -2329,69 +2329,69 @@
         </is>
       </c>
       <c r="H53" s="8" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="12" t="inlineStr">
-        <is>
-          <t>Soportes y bases</t>
-        </is>
-      </c>
-      <c r="B54" s="12" t="inlineStr">
-        <is>
-          <t>Gato Soporte Elevador Moto Rueda Trasera Delantera 350kgs</t>
-        </is>
-      </c>
-      <c r="C54" s="12" t="inlineStr">
-        <is>
-          <t>Negro</t>
-        </is>
-      </c>
-      <c r="D54" s="12" t="inlineStr">
-        <is>
-          <t>GZTYJ-41046N</t>
-        </is>
-      </c>
-      <c r="E54" s="13" t="n">
-        <v>2890</v>
-      </c>
-      <c r="F54" s="14">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Protección</t>
+        </is>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>Protector De Levas Universal Moto ABS Varios Colores - Azul</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>Protectores de levas</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>HP-Q035B2</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="n">
+        <v>890</v>
+      </c>
+      <c r="F54" s="6">
         <f>ROUND(E54*0.9,0)</f>
         <v/>
       </c>
-      <c r="G54" s="12" t="inlineStr">
-        <is>
-          <t>Sin stock</t>
-        </is>
-      </c>
-      <c r="H54" s="12" t="n">
-        <v>0</v>
+      <c r="G54" s="7" t="inlineStr">
+        <is>
+          <t>Con stock</t>
+        </is>
+      </c>
+      <c r="H54" s="4" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="15" t="inlineStr">
         <is>
-          <t>Soportes y bases</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="B55" s="15" t="inlineStr">
         <is>
-          <t>Gato Soporte Elevador Moto Rueda Trasera Delantera 350kgs</t>
+          <t>Protector De Levas Universal Moto ABS Varios Colores - Rojo</t>
         </is>
       </c>
       <c r="C55" s="15" t="inlineStr">
         <is>
-          <t>Rojo</t>
+          <t>Protectores de levas</t>
         </is>
       </c>
       <c r="D55" s="15" t="inlineStr">
         <is>
-          <t>GZTYJ-41046R</t>
+          <t>HP-Q035B3</t>
         </is>
       </c>
       <c r="E55" s="16" t="n">
-        <v>2890</v>
+        <v>890</v>
       </c>
       <c r="F55" s="17">
         <f>ROUND(E55*0.9,0)</f>
@@ -2407,283 +2407,283 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="12" t="inlineStr">
-        <is>
-          <t>Posapiés</t>
-        </is>
-      </c>
-      <c r="B56" s="12" t="inlineStr">
-        <is>
-          <t>Posapies Universales De Aluminio Negro Para Moto</t>
-        </is>
-      </c>
-      <c r="C56" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D56" s="12" t="inlineStr">
-        <is>
-          <t>POSAPIE1</t>
-        </is>
-      </c>
-      <c r="E56" s="13" t="n">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Protección</t>
+        </is>
+      </c>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>Protector De Levas Freno Y Embrague Estilo Fibra De Carbono</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>Protectores de levas</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>HS-30006</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="n">
+        <v>690</v>
+      </c>
+      <c r="F56" s="6">
+        <f>ROUND(E56*0.9,0)</f>
+        <v/>
+      </c>
+      <c r="G56" s="7" t="inlineStr">
+        <is>
+          <t>Con stock</t>
+        </is>
+      </c>
+      <c r="H56" s="4" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="8" t="inlineStr">
+        <is>
+          <t>Protección</t>
+        </is>
+      </c>
+      <c r="B57" s="8" t="inlineStr">
+        <is>
+          <t>Protector De Levas Universal Aluminio Negro (uso deportivo)</t>
+        </is>
+      </c>
+      <c r="C57" s="8" t="inlineStr">
+        <is>
+          <t>Protectores de levas</t>
+        </is>
+      </c>
+      <c r="D57" s="8" t="inlineStr">
+        <is>
+          <t>MELI-MLU1039263040</t>
+        </is>
+      </c>
+      <c r="E57" s="9" t="n">
+        <v>690</v>
+      </c>
+      <c r="F57" s="10">
+        <f>ROUND(E57*0.9,0)</f>
+        <v/>
+      </c>
+      <c r="G57" s="11" t="inlineStr">
+        <is>
+          <t>Con stock</t>
+        </is>
+      </c>
+      <c r="H57" s="8" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>Protección</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>Slider Universal Aluminio Grande Moto Protector Anti Caídas</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>Sliders</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>FSB-002</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="n">
         <v>1290</v>
       </c>
-      <c r="F56" s="14">
-        <f>ROUND(E56*0.9,0)</f>
-        <v/>
-      </c>
-      <c r="G56" s="12" t="inlineStr">
-        <is>
-          <t>Sin stock</t>
-        </is>
-      </c>
-      <c r="H56" s="12" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="15" t="inlineStr">
-        <is>
-          <t>Posapiés</t>
-        </is>
-      </c>
-      <c r="B57" s="15" t="inlineStr">
-        <is>
-          <t>Posapies Aluminio CNC Moto Cross Enduro Antideslizante</t>
-        </is>
-      </c>
-      <c r="C57" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D57" s="15" t="inlineStr">
-        <is>
-          <t>HP-ZJ039</t>
-        </is>
-      </c>
-      <c r="E57" s="16" t="n">
-        <v>1590</v>
-      </c>
-      <c r="F57" s="17">
-        <f>ROUND(E57*0.9,0)</f>
-        <v/>
-      </c>
-      <c r="G57" s="15" t="inlineStr">
-        <is>
-          <t>Sin stock</t>
-        </is>
-      </c>
-      <c r="H57" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="12" t="inlineStr">
-        <is>
-          <t>Escapes</t>
-        </is>
-      </c>
-      <c r="B58" s="12" t="inlineStr">
-        <is>
-          <t>Escape SC Project 51mm Universal Moto</t>
-        </is>
-      </c>
-      <c r="C58" s="12" t="inlineStr">
-        <is>
-          <t>Negro</t>
-        </is>
-      </c>
-      <c r="D58" s="12" t="inlineStr">
-        <is>
-          <t>HP-EXHAUST-GBLACK</t>
-        </is>
-      </c>
-      <c r="E58" s="13" t="n">
-        <v>2490</v>
-      </c>
-      <c r="F58" s="14">
+      <c r="F58" s="6">
         <f>ROUND(E58*0.9,0)</f>
         <v/>
       </c>
-      <c r="G58" s="12" t="inlineStr">
-        <is>
-          <t>Sin stock</t>
-        </is>
-      </c>
-      <c r="H58" s="12" t="n">
-        <v>0</v>
+      <c r="G58" s="7" t="inlineStr">
+        <is>
+          <t>Con stock</t>
+        </is>
+      </c>
+      <c r="H58" s="4" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="15" t="inlineStr">
-        <is>
-          <t>Escapes</t>
-        </is>
-      </c>
-      <c r="B59" s="15" t="inlineStr">
-        <is>
-          <t>Escape SC Project 51mm Universal Moto</t>
-        </is>
-      </c>
-      <c r="C59" s="15" t="inlineStr">
-        <is>
-          <t>Plateado</t>
-        </is>
-      </c>
-      <c r="D59" s="15" t="inlineStr">
-        <is>
-          <t>HP-EXHAUST-GSILVER</t>
-        </is>
-      </c>
-      <c r="E59" s="16" t="n">
-        <v>2190</v>
-      </c>
-      <c r="F59" s="17">
+      <c r="A59" s="8" t="inlineStr">
+        <is>
+          <t>Protección</t>
+        </is>
+      </c>
+      <c r="B59" s="8" t="inlineStr">
+        <is>
+          <t>Slider Universal Aluminio Moto Protector Anti Caídas Naranja</t>
+        </is>
+      </c>
+      <c r="C59" s="8" t="inlineStr">
+        <is>
+          <t>Sliders</t>
+        </is>
+      </c>
+      <c r="D59" s="8" t="inlineStr">
+        <is>
+          <t>FSB-003</t>
+        </is>
+      </c>
+      <c r="E59" s="9" t="n">
+        <v>1290</v>
+      </c>
+      <c r="F59" s="10">
         <f>ROUND(E59*0.9,0)</f>
         <v/>
       </c>
-      <c r="G59" s="15" t="inlineStr">
-        <is>
-          <t>Sin stock</t>
-        </is>
-      </c>
-      <c r="H59" s="15" t="n">
-        <v>0</v>
+      <c r="G59" s="11" t="inlineStr">
+        <is>
+          <t>Con stock</t>
+        </is>
+      </c>
+      <c r="H59" s="8" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="12" t="inlineStr">
-        <is>
-          <t>Escapes</t>
-        </is>
-      </c>
-      <c r="B60" s="12" t="inlineStr">
-        <is>
-          <t>Escape SC Project Boca Inclinada 51mm Negro Universal Moto</t>
-        </is>
-      </c>
-      <c r="C60" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D60" s="12" t="inlineStr">
-        <is>
-          <t>AP-SLANTED01</t>
-        </is>
-      </c>
-      <c r="E60" s="13" t="n">
-        <v>2590</v>
-      </c>
-      <c r="F60" s="14">
+      <c r="A60" s="4" t="inlineStr">
+        <is>
+          <t>Matrícula</t>
+        </is>
+      </c>
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>Porta Matricula Rebatible Placa Patente Moto Rebatible</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>Rebatible</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>CPJ-62001</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="n">
+        <v>1290</v>
+      </c>
+      <c r="F60" s="6">
         <f>ROUND(E60*0.9,0)</f>
         <v/>
       </c>
-      <c r="G60" s="12" t="inlineStr">
-        <is>
-          <t>Sin stock</t>
-        </is>
-      </c>
-      <c r="H60" s="12" t="n">
-        <v>0</v>
+      <c r="G60" s="7" t="inlineStr">
+        <is>
+          <t>Con stock</t>
+        </is>
+      </c>
+      <c r="H60" s="4" t="n">
+        <v>38</v>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="15" t="inlineStr">
-        <is>
-          <t>Escapes</t>
-        </is>
-      </c>
-      <c r="B61" s="15" t="inlineStr">
-        <is>
-          <t>Escape tipo Akrapovic 51mm Universal Moto</t>
-        </is>
-      </c>
-      <c r="C61" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D61" s="15" t="inlineStr">
-        <is>
-          <t>HP-EXHAUST-A</t>
-        </is>
-      </c>
-      <c r="E61" s="16" t="n">
-        <v>3990</v>
-      </c>
-      <c r="F61" s="17">
+      <c r="A61" s="8" t="inlineStr">
+        <is>
+          <t>Matrícula</t>
+        </is>
+      </c>
+      <c r="B61" s="8" t="inlineStr">
+        <is>
+          <t>Porta Matricula Moto Rebatible Compacto Perfil Bajo</t>
+        </is>
+      </c>
+      <c r="C61" s="8" t="inlineStr">
+        <is>
+          <t>Rebatible</t>
+        </is>
+      </c>
+      <c r="D61" s="8" t="inlineStr">
+        <is>
+          <t>PATENTE1</t>
+        </is>
+      </c>
+      <c r="E61" s="9" t="n">
+        <v>890</v>
+      </c>
+      <c r="F61" s="10">
         <f>ROUND(E61*0.9,0)</f>
         <v/>
       </c>
-      <c r="G61" s="15" t="inlineStr">
-        <is>
-          <t>Sin stock</t>
-        </is>
-      </c>
-      <c r="H61" s="15" t="n">
-        <v>0</v>
+      <c r="G61" s="11" t="inlineStr">
+        <is>
+          <t>Con stock</t>
+        </is>
+      </c>
+      <c r="H61" s="8" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="12" t="inlineStr">
-        <is>
-          <t>Escapes</t>
-        </is>
-      </c>
-      <c r="B62" s="12" t="inlineStr">
-        <is>
-          <t>Escape Yoshimura Fibra Carbono Universal Moto Deportivo 51mm</t>
-        </is>
-      </c>
-      <c r="C62" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D62" s="12" t="inlineStr">
-        <is>
-          <t>AP-YOSHIMURA01</t>
-        </is>
-      </c>
-      <c r="E62" s="13" t="n">
-        <v>5890</v>
-      </c>
-      <c r="F62" s="14">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
+          <t>Carenado</t>
+        </is>
+      </c>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>Guardabarros Trasero Universal Moto ABS</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>Guardabarros</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>HP-DB004-B</t>
+        </is>
+      </c>
+      <c r="E62" s="5" t="n">
+        <v>1290</v>
+      </c>
+      <c r="F62" s="6">
         <f>ROUND(E62*0.9,0)</f>
         <v/>
       </c>
-      <c r="G62" s="12" t="inlineStr">
-        <is>
-          <t>Sin stock</t>
-        </is>
-      </c>
-      <c r="H62" s="12" t="n">
-        <v>0</v>
+      <c r="G62" s="7" t="inlineStr">
+        <is>
+          <t>Con stock</t>
+        </is>
+      </c>
+      <c r="H62" s="4" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="15" t="inlineStr">
         <is>
-          <t>Baúles</t>
+          <t>Carenado</t>
         </is>
       </c>
       <c r="B63" s="15" t="inlineStr">
         <is>
-          <t>Baúl Trasero Moto 28L ABS Clásico Seguro Universal Con Llave</t>
+          <t>Deflector Parabrisas Para Moto Universal Transparente</t>
         </is>
       </c>
       <c r="C63" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Parabrisas</t>
         </is>
       </c>
       <c r="D63" s="15" t="inlineStr">
         <is>
-          <t>AP-TAILBOXLED</t>
+          <t>DFB-002</t>
         </is>
       </c>
       <c r="E63" s="16" t="n">
@@ -2705,26 +2705,26 @@
     <row r="64">
       <c r="A64" s="12" t="inlineStr">
         <is>
-          <t>Baúles</t>
+          <t>Eléctrico</t>
         </is>
       </c>
       <c r="B64" s="12" t="inlineStr">
         <is>
-          <t>Baúl Trasero Moto 45L PP Alta Resistencia Universal Con Llave</t>
+          <t>Señaleros LED Finos Universales 12V Para Moto - Amarillo</t>
         </is>
       </c>
       <c r="C64" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Señaleros LED</t>
         </is>
       </c>
       <c r="D64" s="12" t="inlineStr">
         <is>
-          <t>AP-TAILBOXSQ</t>
+          <t>HP-Z0533</t>
         </is>
       </c>
       <c r="E64" s="13" t="n">
-        <v>3990</v>
+        <v>320</v>
       </c>
       <c r="F64" s="14">
         <f>ROUND(E64*0.9,0)</f>
@@ -2739,8 +2739,304 @@
         <v>0</v>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" s="15" t="inlineStr">
+        <is>
+          <t>Eléctrico</t>
+        </is>
+      </c>
+      <c r="B65" s="15" t="inlineStr">
+        <is>
+          <t>Señaleros Led Secuenciales Luz Amarilla Universales Moto Amarillo</t>
+        </is>
+      </c>
+      <c r="C65" s="15" t="inlineStr">
+        <is>
+          <t>Señaleros LED</t>
+        </is>
+      </c>
+      <c r="D65" s="15" t="inlineStr">
+        <is>
+          <t>SEÑAL01</t>
+        </is>
+      </c>
+      <c r="E65" s="16" t="n">
+        <v>350</v>
+      </c>
+      <c r="F65" s="17">
+        <f>ROUND(E65*0.9,0)</f>
+        <v/>
+      </c>
+      <c r="G65" s="15" t="inlineStr">
+        <is>
+          <t>Sin stock</t>
+        </is>
+      </c>
+      <c r="H65" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="12" t="inlineStr">
+        <is>
+          <t>Escapes</t>
+        </is>
+      </c>
+      <c r="B66" s="12" t="inlineStr">
+        <is>
+          <t>Escape SC Project 51mm Universal Moto - Negro</t>
+        </is>
+      </c>
+      <c r="C66" s="12" t="inlineStr">
+        <is>
+          <t>SC Project</t>
+        </is>
+      </c>
+      <c r="D66" s="12" t="inlineStr">
+        <is>
+          <t>HP-EXHAUST-GBLACK</t>
+        </is>
+      </c>
+      <c r="E66" s="13" t="n">
+        <v>2490</v>
+      </c>
+      <c r="F66" s="14">
+        <f>ROUND(E66*0.9,0)</f>
+        <v/>
+      </c>
+      <c r="G66" s="12" t="inlineStr">
+        <is>
+          <t>Sin stock</t>
+        </is>
+      </c>
+      <c r="H66" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="15" t="inlineStr">
+        <is>
+          <t>Escapes</t>
+        </is>
+      </c>
+      <c r="B67" s="15" t="inlineStr">
+        <is>
+          <t>Escape SC Project 51mm Universal Moto - Plateado</t>
+        </is>
+      </c>
+      <c r="C67" s="15" t="inlineStr">
+        <is>
+          <t>SC Project</t>
+        </is>
+      </c>
+      <c r="D67" s="15" t="inlineStr">
+        <is>
+          <t>HP-EXHAUST-GSILVER</t>
+        </is>
+      </c>
+      <c r="E67" s="16" t="n">
+        <v>2190</v>
+      </c>
+      <c r="F67" s="17">
+        <f>ROUND(E67*0.9,0)</f>
+        <v/>
+      </c>
+      <c r="G67" s="15" t="inlineStr">
+        <is>
+          <t>Sin stock</t>
+        </is>
+      </c>
+      <c r="H67" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="12" t="inlineStr">
+        <is>
+          <t>Escapes</t>
+        </is>
+      </c>
+      <c r="B68" s="12" t="inlineStr">
+        <is>
+          <t>Escape SC Project Boca Inclinada 51mm Negro Universal Moto</t>
+        </is>
+      </c>
+      <c r="C68" s="12" t="inlineStr">
+        <is>
+          <t>SC Project</t>
+        </is>
+      </c>
+      <c r="D68" s="12" t="inlineStr">
+        <is>
+          <t>AP-SLANTED01</t>
+        </is>
+      </c>
+      <c r="E68" s="13" t="n">
+        <v>2590</v>
+      </c>
+      <c r="F68" s="14">
+        <f>ROUND(E68*0.9,0)</f>
+        <v/>
+      </c>
+      <c r="G68" s="12" t="inlineStr">
+        <is>
+          <t>Sin stock</t>
+        </is>
+      </c>
+      <c r="H68" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="15" t="inlineStr">
+        <is>
+          <t>Escapes</t>
+        </is>
+      </c>
+      <c r="B69" s="15" t="inlineStr">
+        <is>
+          <t>Escape Tipo Akrapovic 51mm Universal Moto</t>
+        </is>
+      </c>
+      <c r="C69" s="15" t="inlineStr">
+        <is>
+          <t>Akrapovic</t>
+        </is>
+      </c>
+      <c r="D69" s="15" t="inlineStr">
+        <is>
+          <t>HP-EXHAUST-A</t>
+        </is>
+      </c>
+      <c r="E69" s="16" t="n">
+        <v>3990</v>
+      </c>
+      <c r="F69" s="17">
+        <f>ROUND(E69*0.9,0)</f>
+        <v/>
+      </c>
+      <c r="G69" s="15" t="inlineStr">
+        <is>
+          <t>Sin stock</t>
+        </is>
+      </c>
+      <c r="H69" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="12" t="inlineStr">
+        <is>
+          <t>Escapes</t>
+        </is>
+      </c>
+      <c r="B70" s="12" t="inlineStr">
+        <is>
+          <t>Escape Yoshimura Fibra Carbono Universal Moto Deportivo 51mm</t>
+        </is>
+      </c>
+      <c r="C70" s="12" t="inlineStr">
+        <is>
+          <t>Yoshimura</t>
+        </is>
+      </c>
+      <c r="D70" s="12" t="inlineStr">
+        <is>
+          <t>AP-YOSHIMURA01</t>
+        </is>
+      </c>
+      <c r="E70" s="13" t="n">
+        <v>5890</v>
+      </c>
+      <c r="F70" s="14">
+        <f>ROUND(E70*0.9,0)</f>
+        <v/>
+      </c>
+      <c r="G70" s="12" t="inlineStr">
+        <is>
+          <t>Sin stock</t>
+        </is>
+      </c>
+      <c r="H70" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="15" t="inlineStr">
+        <is>
+          <t>Baúles</t>
+        </is>
+      </c>
+      <c r="B71" s="15" t="inlineStr">
+        <is>
+          <t>Baúl Trasero Moto 28L ABS Clásico Seguro Universal Con Llave</t>
+        </is>
+      </c>
+      <c r="C71" s="15" t="inlineStr">
+        <is>
+          <t>Traseros</t>
+        </is>
+      </c>
+      <c r="D71" s="15" t="inlineStr">
+        <is>
+          <t>AP-TAILBOXLED</t>
+        </is>
+      </c>
+      <c r="E71" s="16" t="n">
+        <v>1750</v>
+      </c>
+      <c r="F71" s="17">
+        <f>ROUND(E71*0.9,0)</f>
+        <v/>
+      </c>
+      <c r="G71" s="15" t="inlineStr">
+        <is>
+          <t>Sin stock</t>
+        </is>
+      </c>
+      <c r="H71" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="12" t="inlineStr">
+        <is>
+          <t>Baúles</t>
+        </is>
+      </c>
+      <c r="B72" s="12" t="inlineStr">
+        <is>
+          <t>Baúl Trasero Moto 45L PP Alta Resistencia Universal Con Llave</t>
+        </is>
+      </c>
+      <c r="C72" s="12" t="inlineStr">
+        <is>
+          <t>Traseros</t>
+        </is>
+      </c>
+      <c r="D72" s="12" t="inlineStr">
+        <is>
+          <t>AP-TAILBOXSQ</t>
+        </is>
+      </c>
+      <c r="E72" s="13" t="n">
+        <v>3990</v>
+      </c>
+      <c r="F72" s="14">
+        <f>ROUND(E72*0.9,0)</f>
+        <v/>
+      </c>
+      <c r="G72" s="12" t="inlineStr">
+        <is>
+          <t>Sin stock</t>
+        </is>
+      </c>
+      <c r="H72" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:H64"/>
+  <autoFilter ref="A5:H72"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Lista de precios: sin los extensores de rosca
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015XoTitFW4NKs6Tkz8h27S9
</commit_message>
<xml_diff>
--- a/docs/meta-ia/lista-precios-martinez-motos.xlsx
+++ b/docs/meta-ia/lista-precios-martinez-motos.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lista de precios" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Lista de precios'!$A$5:$H$72</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Lista de precios'!$A$5:$H$56</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Lista de precios'!$5:$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H72"/>
+  <dimension ref="A1:H56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -744,26 +744,26 @@
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>Espejos</t>
+          <t>Soportes y bases</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>Extensor Espejo Moto Rosca 8mm Int/Ext Horario Universal</t>
+          <t>Soporte Celular Moto Universal Manillar Negro Ajustable</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>Extensores</t>
+          <t>Soportes de celular</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>EXT-ESP-8F-8F-001</t>
+          <t>SOP-CEL-MAN-001</t>
         </is>
       </c>
       <c r="E11" s="9" t="n">
-        <v>100</v>
+        <v>490</v>
       </c>
       <c r="F11" s="10">
         <f>ROUND(E11*0.9,0)</f>
@@ -775,32 +775,32 @@
         </is>
       </c>
       <c r="H11" s="8" t="n">
-        <v>10</v>
+        <v>87</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Espejos</t>
+          <t>Soportes y bases</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Extensor Espejo Moto Rosca 8mm Int/Ext Antihorario Univ</t>
+          <t>Soporte Celular Moto Universal Espejo Negro Ajustable</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Extensores</t>
+          <t>Soportes de celular</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>EXT-ESP-8R-8R-001</t>
+          <t>SOP-CEL-ESP-001</t>
         </is>
       </c>
       <c r="E12" s="5" t="n">
-        <v>100</v>
+        <v>490</v>
       </c>
       <c r="F12" s="6">
         <f>ROUND(E12*0.9,0)</f>
@@ -812,32 +812,32 @@
         </is>
       </c>
       <c r="H12" s="4" t="n">
-        <v>10</v>
+        <v>89</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>Espejos</t>
+          <t>Soportes y bases</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Extensor Espejo Moto Rosca 8mm Int Hor / Ext Antihor</t>
+          <t>Extensor De Pie Pata Lateral Moto Bicicleta Base Soporte Negro</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>Extensores</t>
+          <t>Pata lateral</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>EXT-ESP-8F-8R-001</t>
+          <t>YTLY-30</t>
         </is>
       </c>
       <c r="E13" s="9" t="n">
-        <v>100</v>
+        <v>274</v>
       </c>
       <c r="F13" s="10">
         <f>ROUND(E13*0.9,0)</f>
@@ -849,106 +849,106 @@
         </is>
       </c>
       <c r="H13" s="8" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>Espejos</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>Extensor Espejo Moto Rosca 8mm Int Antihor / Ext Hor</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>Extensores</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>EXT-ESP-8R-8F-001</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="F14" s="6">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>Soportes y bases</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>Gato Soporte Elevador Moto Rueda Trasera Delantera 350kgs - Negro</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="inlineStr">
+        <is>
+          <t>Gatos elevadores</t>
+        </is>
+      </c>
+      <c r="D14" s="12" t="inlineStr">
+        <is>
+          <t>GZTYJ-41046N</t>
+        </is>
+      </c>
+      <c r="E14" s="13" t="n">
+        <v>2890</v>
+      </c>
+      <c r="F14" s="14">
         <f>ROUND(E14*0.9,0)</f>
         <v/>
       </c>
-      <c r="G14" s="7" t="inlineStr">
-        <is>
-          <t>Con stock</t>
-        </is>
-      </c>
-      <c r="H14" s="4" t="n">
-        <v>10</v>
+      <c r="G14" s="12" t="inlineStr">
+        <is>
+          <t>Sin stock</t>
+        </is>
+      </c>
+      <c r="H14" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
-        <is>
-          <t>Espejos</t>
-        </is>
-      </c>
-      <c r="B15" s="8" t="inlineStr">
-        <is>
-          <t>Extensor Espejo Moto Rosca 8mm Int Hor / 10mm Ext Hor</t>
-        </is>
-      </c>
-      <c r="C15" s="8" t="inlineStr">
-        <is>
-          <t>Extensores</t>
-        </is>
-      </c>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>EXT-ESP-8F-10F-001</t>
-        </is>
-      </c>
-      <c r="E15" s="9" t="n">
-        <v>100</v>
-      </c>
-      <c r="F15" s="10">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>Soportes y bases</t>
+        </is>
+      </c>
+      <c r="B15" s="15" t="inlineStr">
+        <is>
+          <t>Gato Soporte Elevador Moto Rueda Trasera Delantera 350kgs - Rojo</t>
+        </is>
+      </c>
+      <c r="C15" s="15" t="inlineStr">
+        <is>
+          <t>Gatos elevadores</t>
+        </is>
+      </c>
+      <c r="D15" s="15" t="inlineStr">
+        <is>
+          <t>GZTYJ-41046R</t>
+        </is>
+      </c>
+      <c r="E15" s="16" t="n">
+        <v>2890</v>
+      </c>
+      <c r="F15" s="17">
         <f>ROUND(E15*0.9,0)</f>
         <v/>
       </c>
-      <c r="G15" s="11" t="inlineStr">
-        <is>
-          <t>Con stock</t>
-        </is>
-      </c>
-      <c r="H15" s="8" t="n">
-        <v>10</v>
+      <c r="G15" s="15" t="inlineStr">
+        <is>
+          <t>Sin stock</t>
+        </is>
+      </c>
+      <c r="H15" s="15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Espejos</t>
+          <t>Puños</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Extensor Espejo Moto Rosca 8mm Int Hor / 10mm Ext Antihor</t>
+          <t>Puños Domino Para Moto Manubrio Goma Antideslizante Negro</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Extensores</t>
+          <t>Domino</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>EXT-ESP-8F-10R-001</t>
+          <t>DOM00</t>
         </is>
       </c>
       <c r="E16" s="5" t="n">
-        <v>100</v>
+        <v>450</v>
       </c>
       <c r="F16" s="6">
         <f>ROUND(E16*0.9,0)</f>
@@ -960,32 +960,32 @@
         </is>
       </c>
       <c r="H16" s="4" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>Espejos</t>
+          <t>Puños</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>Extensor Espejo Moto Rosca 8mm Int Antihor / 10mm Ext</t>
+          <t>Puños Domino Para Moto Manubrio Goma Antideslizante Rojo</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>Extensores</t>
+          <t>Domino</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>EXT-ESP-8R-10F-001</t>
+          <t>DOM01</t>
         </is>
       </c>
       <c r="E17" s="9" t="n">
-        <v>100</v>
+        <v>450</v>
       </c>
       <c r="F17" s="10">
         <f>ROUND(E17*0.9,0)</f>
@@ -997,32 +997,32 @@
         </is>
       </c>
       <c r="H17" s="8" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Espejos</t>
+          <t>Puños</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Extensor Espejo Moto Rosca 8mm Int/10mm Ext Antihorario</t>
+          <t>Puños Domino Para Moto Manubrio Goma Antideslizante Azul</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Extensores</t>
+          <t>Domino</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>EXT-ESP-8R-10R-001</t>
+          <t>DOM02</t>
         </is>
       </c>
       <c r="E18" s="5" t="n">
-        <v>100</v>
+        <v>450</v>
       </c>
       <c r="F18" s="6">
         <f>ROUND(E18*0.9,0)</f>
@@ -1034,32 +1034,32 @@
         </is>
       </c>
       <c r="H18" s="4" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>Espejos</t>
+          <t>Puños</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>Extensor Espejo Moto Rosca 10mm Int/Ext Horario Universal</t>
+          <t>Puños Domino Para Moto Manubrio Goma Antideslizante Naranja</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>Extensores</t>
+          <t>Domino</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>EXT-ESP-10F-10F-001</t>
+          <t>DOM03</t>
         </is>
       </c>
       <c r="E19" s="9" t="n">
-        <v>100</v>
+        <v>450</v>
       </c>
       <c r="F19" s="10">
         <f>ROUND(E19*0.9,0)</f>
@@ -1071,32 +1071,32 @@
         </is>
       </c>
       <c r="H19" s="8" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Espejos</t>
+          <t>Puños</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Extensor Espejo Moto Rosca 10mm Int/Ext Antihorario Univ</t>
+          <t>Puños Domino Para Moto Manubrio Goma Antideslizante Verde</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Extensores</t>
+          <t>Domino</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>EXT-ESP-10R-10R-001</t>
+          <t>DOM04</t>
         </is>
       </c>
       <c r="E20" s="5" t="n">
-        <v>100</v>
+        <v>450</v>
       </c>
       <c r="F20" s="6">
         <f>ROUND(E20*0.9,0)</f>
@@ -1108,32 +1108,32 @@
         </is>
       </c>
       <c r="H20" s="4" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>Espejos</t>
+          <t>Puños</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>Extensor Espejo Moto Rosca 10mm Int Hor / Ext Antihor</t>
+          <t>Puños Universales Antideslizantes Con Contrapesos Anticaídas Negro</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>Extensores</t>
+          <t>Con contrapeso</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>EXT-ESP-10F-10R-001</t>
+          <t>PUNBLACK</t>
         </is>
       </c>
       <c r="E21" s="9" t="n">
-        <v>100</v>
+        <v>990</v>
       </c>
       <c r="F21" s="10">
         <f>ROUND(E21*0.9,0)</f>
@@ -1145,32 +1145,32 @@
         </is>
       </c>
       <c r="H21" s="8" t="n">
-        <v>10</v>
+        <v>21</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>Espejos</t>
+          <t>Puños</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Extensor Espejo Moto Rosca 10mm Int Antihor / Ext Hor</t>
+          <t>Puños Universales Antideslizantes Con Contrapesos Anticaídas Dorado</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Extensores</t>
+          <t>Con contrapeso</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>EXT-ESP-10R-10F-001</t>
+          <t>PUNYELLOW</t>
         </is>
       </c>
       <c r="E22" s="5" t="n">
-        <v>100</v>
+        <v>990</v>
       </c>
       <c r="F22" s="6">
         <f>ROUND(E22*0.9,0)</f>
@@ -1182,106 +1182,106 @@
         </is>
       </c>
       <c r="H22" s="4" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="inlineStr">
-        <is>
-          <t>Espejos</t>
-        </is>
-      </c>
-      <c r="B23" s="8" t="inlineStr">
-        <is>
-          <t>Extensor Espejo Moto Rosca 10mm Int Hor / 8mm Ext Hor</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="inlineStr">
-        <is>
-          <t>Extensores</t>
-        </is>
-      </c>
-      <c r="D23" s="8" t="inlineStr">
-        <is>
-          <t>EXT-ESP-10F-8F-001</t>
-        </is>
-      </c>
-      <c r="E23" s="9" t="n">
-        <v>100</v>
-      </c>
-      <c r="F23" s="10">
+      <c r="A23" s="15" t="inlineStr">
+        <is>
+          <t>Puños</t>
+        </is>
+      </c>
+      <c r="B23" s="15" t="inlineStr">
+        <is>
+          <t>Puños Universales Antideslizantes Con Contrapesos Anticaídas Rojo</t>
+        </is>
+      </c>
+      <c r="C23" s="15" t="inlineStr">
+        <is>
+          <t>Con contrapeso</t>
+        </is>
+      </c>
+      <c r="D23" s="15" t="inlineStr">
+        <is>
+          <t>PUNRED</t>
+        </is>
+      </c>
+      <c r="E23" s="16" t="n">
+        <v>990</v>
+      </c>
+      <c r="F23" s="17">
         <f>ROUND(E23*0.9,0)</f>
         <v/>
       </c>
-      <c r="G23" s="11" t="inlineStr">
-        <is>
-          <t>Con stock</t>
-        </is>
-      </c>
-      <c r="H23" s="8" t="n">
-        <v>10</v>
+      <c r="G23" s="15" t="inlineStr">
+        <is>
+          <t>Sin stock</t>
+        </is>
+      </c>
+      <c r="H23" s="15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>Espejos</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>Extensor Espejo Moto Rosca 10mm Int Hor / 8mm Ext Antihor</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>Extensores</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>EXT-ESP-10F-8R-001</t>
-        </is>
-      </c>
-      <c r="E24" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="F24" s="6">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>Puños</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>Puños Universales Antideslizantes Con Contrapesos Anticaídas Naranja</t>
+        </is>
+      </c>
+      <c r="C24" s="12" t="inlineStr">
+        <is>
+          <t>Con contrapeso</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>PUNORGANG</t>
+        </is>
+      </c>
+      <c r="E24" s="13" t="n">
+        <v>990</v>
+      </c>
+      <c r="F24" s="14">
         <f>ROUND(E24*0.9,0)</f>
         <v/>
       </c>
-      <c r="G24" s="7" t="inlineStr">
-        <is>
-          <t>Con stock</t>
-        </is>
-      </c>
-      <c r="H24" s="4" t="n">
-        <v>10</v>
+      <c r="G24" s="12" t="inlineStr">
+        <is>
+          <t>Sin stock</t>
+        </is>
+      </c>
+      <c r="H24" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>Espejos</t>
+          <t>Manillares</t>
         </is>
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>Extensor Espejo Moto Rosca 10mm Int Antihor / 8mm Ext</t>
+          <t>Manillar Universal Aluminio Para Moto 22mm - Negro</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>Extensores</t>
+          <t>Universal 7/8</t>
         </is>
       </c>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t>EXT-ESP-10R-8F-001</t>
+          <t>HP-CB0381</t>
         </is>
       </c>
       <c r="E25" s="9" t="n">
-        <v>100</v>
+        <v>1190</v>
       </c>
       <c r="F25" s="10">
         <f>ROUND(E25*0.9,0)</f>
@@ -1293,32 +1293,32 @@
         </is>
       </c>
       <c r="H25" s="8" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>Espejos</t>
+          <t>Manillares</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Extensor Espejo Moto Rosca 10mm Int/8mm Ext Antihorario</t>
+          <t>Manillar Universal Aluminio Para Moto 22mm - Blanco</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Extensores</t>
+          <t>Universal 7/8</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>EXT-ESP-10R-8R-001</t>
+          <t>HP-CB0382</t>
         </is>
       </c>
       <c r="E26" s="5" t="n">
-        <v>100</v>
+        <v>1190</v>
       </c>
       <c r="F26" s="6">
         <f>ROUND(E26*0.9,0)</f>
@@ -1330,32 +1330,32 @@
         </is>
       </c>
       <c r="H26" s="4" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>Soportes y bases</t>
+          <t>Manillares</t>
         </is>
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>Soporte Celular Moto Universal Manillar Negro Ajustable</t>
+          <t>Manillar Universal Aluminio Para Moto 22mm - Amarillo</t>
         </is>
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>Soportes de celular</t>
+          <t>Universal 7/8</t>
         </is>
       </c>
       <c r="D27" s="8" t="inlineStr">
         <is>
-          <t>SOP-CEL-MAN-001</t>
+          <t>HP-CB0383</t>
         </is>
       </c>
       <c r="E27" s="9" t="n">
-        <v>490</v>
+        <v>1190</v>
       </c>
       <c r="F27" s="10">
         <f>ROUND(E27*0.9,0)</f>
@@ -1367,32 +1367,32 @@
         </is>
       </c>
       <c r="H27" s="8" t="n">
-        <v>87</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>Soportes y bases</t>
+          <t>Manillares</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Soporte Celular Moto Universal Espejo Negro Ajustable</t>
+          <t>Manillar Universal Aluminio Para Moto 22mm - Azul</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Soportes de celular</t>
+          <t>Universal 7/8</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>SOP-CEL-ESP-001</t>
+          <t>HP-CB0384</t>
         </is>
       </c>
       <c r="E28" s="5" t="n">
-        <v>490</v>
+        <v>1190</v>
       </c>
       <c r="F28" s="6">
         <f>ROUND(E28*0.9,0)</f>
@@ -1404,32 +1404,32 @@
         </is>
       </c>
       <c r="H28" s="4" t="n">
-        <v>89</v>
+        <v>3</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>Soportes y bases</t>
+          <t>Manillares</t>
         </is>
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>Extensor De Pie Pata Lateral Moto Bicicleta Base Soporte Negro</t>
+          <t>Manillar Universal Aluminio Para Moto 22mm - Rojo</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>Pata lateral</t>
+          <t>Universal 7/8</t>
         </is>
       </c>
       <c r="D29" s="8" t="inlineStr">
         <is>
-          <t>YTLY-30</t>
+          <t>HP-CB0385</t>
         </is>
       </c>
       <c r="E29" s="9" t="n">
-        <v>274</v>
+        <v>1190</v>
       </c>
       <c r="F29" s="10">
         <f>ROUND(E29*0.9,0)</f>
@@ -1441,106 +1441,106 @@
         </is>
       </c>
       <c r="H29" s="8" t="n">
-        <v>14</v>
+        <v>5</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="12" t="inlineStr">
-        <is>
-          <t>Soportes y bases</t>
-        </is>
-      </c>
-      <c r="B30" s="12" t="inlineStr">
-        <is>
-          <t>Gato Soporte Elevador Moto Rueda Trasera Delantera 350kgs - Negro</t>
-        </is>
-      </c>
-      <c r="C30" s="12" t="inlineStr">
-        <is>
-          <t>Gatos elevadores</t>
-        </is>
-      </c>
-      <c r="D30" s="12" t="inlineStr">
-        <is>
-          <t>GZTYJ-41046N</t>
-        </is>
-      </c>
-      <c r="E30" s="13" t="n">
-        <v>2890</v>
-      </c>
-      <c r="F30" s="14">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Manillares</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Manillar Moto Universal 7/8 22mm Alto Negro Antideslizante</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>MAN-78-V2-NEG-001</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="n">
+        <v>690</v>
+      </c>
+      <c r="F30" s="6">
         <f>ROUND(E30*0.9,0)</f>
         <v/>
       </c>
-      <c r="G30" s="12" t="inlineStr">
-        <is>
-          <t>Sin stock</t>
-        </is>
-      </c>
-      <c r="H30" s="12" t="n">
-        <v>0</v>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>Con stock</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="15" t="inlineStr">
-        <is>
-          <t>Soportes y bases</t>
-        </is>
-      </c>
-      <c r="B31" s="15" t="inlineStr">
-        <is>
-          <t>Gato Soporte Elevador Moto Rueda Trasera Delantera 350kgs - Rojo</t>
-        </is>
-      </c>
-      <c r="C31" s="15" t="inlineStr">
-        <is>
-          <t>Gatos elevadores</t>
-        </is>
-      </c>
-      <c r="D31" s="15" t="inlineStr">
-        <is>
-          <t>GZTYJ-41046R</t>
-        </is>
-      </c>
-      <c r="E31" s="16" t="n">
-        <v>2890</v>
-      </c>
-      <c r="F31" s="17">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>Manillares</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>Manillar Moto Universal 7/8 22mm Alto Plateado Antideslizante</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>MAN-78-V2-PLA-001</t>
+        </is>
+      </c>
+      <c r="E31" s="9" t="n">
+        <v>690</v>
+      </c>
+      <c r="F31" s="10">
         <f>ROUND(E31*0.9,0)</f>
         <v/>
       </c>
-      <c r="G31" s="15" t="inlineStr">
-        <is>
-          <t>Sin stock</t>
-        </is>
-      </c>
-      <c r="H31" s="15" t="n">
-        <v>0</v>
+      <c r="G31" s="11" t="inlineStr">
+        <is>
+          <t>Con stock</t>
+        </is>
+      </c>
+      <c r="H31" s="8" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>Puños</t>
+          <t>Manillares</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Puños Domino Para Moto Manubrio Goma Antideslizante Negro</t>
+          <t>Manillar Café Racer Universal 7/8 22mm Recto Negro</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Domino</t>
+          <t>Café Racer</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>DOM00</t>
+          <t>MAN-78-V3-NEG-001</t>
         </is>
       </c>
       <c r="E32" s="5" t="n">
-        <v>450</v>
+        <v>890</v>
       </c>
       <c r="F32" s="6">
         <f>ROUND(E32*0.9,0)</f>
@@ -1552,32 +1552,32 @@
         </is>
       </c>
       <c r="H32" s="4" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>Puños</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>Puños Domino Para Moto Manubrio Goma Antideslizante Rojo</t>
+          <t>Guardamanos Protector Puños Moto Enduro Cross ABS - Negro</t>
         </is>
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>Domino</t>
+          <t>Guardamanos</t>
         </is>
       </c>
       <c r="D33" s="8" t="inlineStr">
         <is>
-          <t>DOM01</t>
+          <t>HP-Q0211</t>
         </is>
       </c>
       <c r="E33" s="9" t="n">
-        <v>450</v>
+        <v>690</v>
       </c>
       <c r="F33" s="10">
         <f>ROUND(E33*0.9,0)</f>
@@ -1589,32 +1589,32 @@
         </is>
       </c>
       <c r="H33" s="8" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>Puños</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Puños Domino Para Moto Manubrio Goma Antideslizante Azul</t>
+          <t>Guardamanos Protector Puños Moto Enduro Cross ABS - Azul</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Domino</t>
+          <t>Guardamanos</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>DOM02</t>
+          <t>HP-Q0212</t>
         </is>
       </c>
       <c r="E34" s="5" t="n">
-        <v>450</v>
+        <v>690</v>
       </c>
       <c r="F34" s="6">
         <f>ROUND(E34*0.9,0)</f>
@@ -1632,26 +1632,26 @@
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>Puños</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>Puños Domino Para Moto Manubrio Goma Antideslizante Naranja</t>
+          <t>Guardamanos Protector Puños Moto Enduro Cross ABS - Rojo</t>
         </is>
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>Domino</t>
+          <t>Guardamanos</t>
         </is>
       </c>
       <c r="D35" s="8" t="inlineStr">
         <is>
-          <t>DOM03</t>
+          <t>HP-Q0213</t>
         </is>
       </c>
       <c r="E35" s="9" t="n">
-        <v>450</v>
+        <v>690</v>
       </c>
       <c r="F35" s="10">
         <f>ROUND(E35*0.9,0)</f>
@@ -1663,32 +1663,32 @@
         </is>
       </c>
       <c r="H35" s="8" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>Puños</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Puños Domino Para Moto Manubrio Goma Antideslizante Verde</t>
+          <t>Guardamanos Moto Con Señalero LED Integrado Negro</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Domino</t>
+          <t>Guardamanos</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>DOM04</t>
+          <t>HP-HS010</t>
         </is>
       </c>
       <c r="E36" s="5" t="n">
-        <v>450</v>
+        <v>990</v>
       </c>
       <c r="F36" s="6">
         <f>ROUND(E36*0.9,0)</f>
@@ -1700,32 +1700,32 @@
         </is>
       </c>
       <c r="H36" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>Puños</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="B37" s="8" t="inlineStr">
         <is>
-          <t>Puños Universales Antideslizantes Con Contrapesos Anticaídas Negro</t>
+          <t>Protector De Levas Universal Moto ABS Varios Colores - Negro</t>
         </is>
       </c>
       <c r="C37" s="8" t="inlineStr">
         <is>
-          <t>Con contrapeso</t>
+          <t>Protectores de levas</t>
         </is>
       </c>
       <c r="D37" s="8" t="inlineStr">
         <is>
-          <t>PUNBLACK</t>
+          <t>HP-Q035B1</t>
         </is>
       </c>
       <c r="E37" s="9" t="n">
-        <v>990</v>
+        <v>890</v>
       </c>
       <c r="F37" s="10">
         <f>ROUND(E37*0.9,0)</f>
@@ -1737,32 +1737,32 @@
         </is>
       </c>
       <c r="H37" s="8" t="n">
-        <v>21</v>
+        <v>10</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>Puños</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Puños Universales Antideslizantes Con Contrapesos Anticaídas Dorado</t>
+          <t>Protector De Levas Universal Moto ABS Varios Colores - Azul</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Con contrapeso</t>
+          <t>Protectores de levas</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>PUNYELLOW</t>
+          <t>HP-Q035B2</t>
         </is>
       </c>
       <c r="E38" s="5" t="n">
-        <v>990</v>
+        <v>890</v>
       </c>
       <c r="F38" s="6">
         <f>ROUND(E38*0.9,0)</f>
@@ -1774,32 +1774,32 @@
         </is>
       </c>
       <c r="H38" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="15" t="inlineStr">
         <is>
-          <t>Puños</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="B39" s="15" t="inlineStr">
         <is>
-          <t>Puños Universales Antideslizantes Con Contrapesos Anticaídas Rojo</t>
+          <t>Protector De Levas Universal Moto ABS Varios Colores - Rojo</t>
         </is>
       </c>
       <c r="C39" s="15" t="inlineStr">
         <is>
-          <t>Con contrapeso</t>
+          <t>Protectores de levas</t>
         </is>
       </c>
       <c r="D39" s="15" t="inlineStr">
         <is>
-          <t>PUNRED</t>
+          <t>HP-Q035B3</t>
         </is>
       </c>
       <c r="E39" s="16" t="n">
-        <v>990</v>
+        <v>890</v>
       </c>
       <c r="F39" s="17">
         <f>ROUND(E39*0.9,0)</f>
@@ -1815,65 +1815,65 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="12" t="inlineStr">
-        <is>
-          <t>Puños</t>
-        </is>
-      </c>
-      <c r="B40" s="12" t="inlineStr">
-        <is>
-          <t>Puños Universales Antideslizantes Con Contrapesos Anticaídas Naranja</t>
-        </is>
-      </c>
-      <c r="C40" s="12" t="inlineStr">
-        <is>
-          <t>Con contrapeso</t>
-        </is>
-      </c>
-      <c r="D40" s="12" t="inlineStr">
-        <is>
-          <t>PUNORGANG</t>
-        </is>
-      </c>
-      <c r="E40" s="13" t="n">
-        <v>990</v>
-      </c>
-      <c r="F40" s="14">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Protección</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>Protector De Levas Freno Y Embrague Estilo Fibra De Carbono</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>Protectores de levas</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>HS-30006</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="n">
+        <v>690</v>
+      </c>
+      <c r="F40" s="6">
         <f>ROUND(E40*0.9,0)</f>
         <v/>
       </c>
-      <c r="G40" s="12" t="inlineStr">
-        <is>
-          <t>Sin stock</t>
-        </is>
-      </c>
-      <c r="H40" s="12" t="n">
-        <v>0</v>
+      <c r="G40" s="7" t="inlineStr">
+        <is>
+          <t>Con stock</t>
+        </is>
+      </c>
+      <c r="H40" s="4" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
         <is>
-          <t>Manillares</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="B41" s="8" t="inlineStr">
         <is>
-          <t>Manillar Universal Aluminio Para Moto 22mm - Negro</t>
+          <t>Protector De Levas Universal Aluminio Negro (uso deportivo)</t>
         </is>
       </c>
       <c r="C41" s="8" t="inlineStr">
         <is>
-          <t>Universal 7/8</t>
+          <t>Protectores de levas</t>
         </is>
       </c>
       <c r="D41" s="8" t="inlineStr">
         <is>
-          <t>HP-CB0381</t>
+          <t>MELI-MLU1039263040</t>
         </is>
       </c>
       <c r="E41" s="9" t="n">
-        <v>1190</v>
+        <v>690</v>
       </c>
       <c r="F41" s="10">
         <f>ROUND(E41*0.9,0)</f>
@@ -1885,32 +1885,32 @@
         </is>
       </c>
       <c r="H41" s="8" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>Manillares</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>Manillar Universal Aluminio Para Moto 22mm - Blanco</t>
+          <t>Slider Universal Aluminio Grande Moto Protector Anti Caídas</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Universal 7/8</t>
+          <t>Sliders</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>HP-CB0382</t>
+          <t>FSB-002</t>
         </is>
       </c>
       <c r="E42" s="5" t="n">
-        <v>1190</v>
+        <v>1290</v>
       </c>
       <c r="F42" s="6">
         <f>ROUND(E42*0.9,0)</f>
@@ -1922,32 +1922,32 @@
         </is>
       </c>
       <c r="H42" s="4" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t>Manillares</t>
+          <t>Protección</t>
         </is>
       </c>
       <c r="B43" s="8" t="inlineStr">
         <is>
-          <t>Manillar Universal Aluminio Para Moto 22mm - Amarillo</t>
+          <t>Slider Universal Aluminio Moto Protector Anti Caídas Naranja</t>
         </is>
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t>Universal 7/8</t>
+          <t>Sliders</t>
         </is>
       </c>
       <c r="D43" s="8" t="inlineStr">
         <is>
-          <t>HP-CB0383</t>
+          <t>FSB-003</t>
         </is>
       </c>
       <c r="E43" s="9" t="n">
-        <v>1190</v>
+        <v>1290</v>
       </c>
       <c r="F43" s="10">
         <f>ROUND(E43*0.9,0)</f>
@@ -1965,26 +1965,26 @@
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>Manillares</t>
+          <t>Matrícula</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>Manillar Universal Aluminio Para Moto 22mm - Azul</t>
+          <t>Porta Matricula Rebatible Placa Patente Moto Rebatible</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Universal 7/8</t>
+          <t>Rebatible</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>HP-CB0384</t>
+          <t>CPJ-62001</t>
         </is>
       </c>
       <c r="E44" s="5" t="n">
-        <v>1190</v>
+        <v>1290</v>
       </c>
       <c r="F44" s="6">
         <f>ROUND(E44*0.9,0)</f>
@@ -1996,32 +1996,32 @@
         </is>
       </c>
       <c r="H44" s="4" t="n">
-        <v>3</v>
+        <v>38</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>Manillares</t>
+          <t>Matrícula</t>
         </is>
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>Manillar Universal Aluminio Para Moto 22mm - Rojo</t>
+          <t>Porta Matricula Moto Rebatible Compacto Perfil Bajo</t>
         </is>
       </c>
       <c r="C45" s="8" t="inlineStr">
         <is>
-          <t>Universal 7/8</t>
+          <t>Rebatible</t>
         </is>
       </c>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>HP-CB0385</t>
+          <t>PATENTE1</t>
         </is>
       </c>
       <c r="E45" s="9" t="n">
-        <v>1190</v>
+        <v>890</v>
       </c>
       <c r="F45" s="10">
         <f>ROUND(E45*0.9,0)</f>
@@ -2033,32 +2033,32 @@
         </is>
       </c>
       <c r="H45" s="8" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>Manillares</t>
+          <t>Carenado</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>Manillar Moto Universal 7/8 22mm Alto Negro Antideslizante</t>
+          <t>Guardabarros Trasero Universal Moto ABS</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Alto</t>
+          <t>Guardabarros</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>MAN-78-V2-NEG-001</t>
+          <t>HP-DB004-B</t>
         </is>
       </c>
       <c r="E46" s="5" t="n">
-        <v>690</v>
+        <v>1290</v>
       </c>
       <c r="F46" s="6">
         <f>ROUND(E46*0.9,0)</f>
@@ -2070,328 +2070,328 @@
         </is>
       </c>
       <c r="H46" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="8" t="inlineStr">
-        <is>
-          <t>Manillares</t>
-        </is>
-      </c>
-      <c r="B47" s="8" t="inlineStr">
-        <is>
-          <t>Manillar Moto Universal 7/8 22mm Alto Plateado Antideslizante</t>
-        </is>
-      </c>
-      <c r="C47" s="8" t="inlineStr">
-        <is>
-          <t>Alto</t>
-        </is>
-      </c>
-      <c r="D47" s="8" t="inlineStr">
-        <is>
-          <t>MAN-78-V2-PLA-001</t>
-        </is>
-      </c>
-      <c r="E47" s="9" t="n">
-        <v>690</v>
-      </c>
-      <c r="F47" s="10">
+      <c r="A47" s="15" t="inlineStr">
+        <is>
+          <t>Carenado</t>
+        </is>
+      </c>
+      <c r="B47" s="15" t="inlineStr">
+        <is>
+          <t>Deflector Parabrisas Para Moto Universal Transparente</t>
+        </is>
+      </c>
+      <c r="C47" s="15" t="inlineStr">
+        <is>
+          <t>Parabrisas</t>
+        </is>
+      </c>
+      <c r="D47" s="15" t="inlineStr">
+        <is>
+          <t>DFB-002</t>
+        </is>
+      </c>
+      <c r="E47" s="16" t="n">
+        <v>1750</v>
+      </c>
+      <c r="F47" s="17">
         <f>ROUND(E47*0.9,0)</f>
         <v/>
       </c>
-      <c r="G47" s="11" t="inlineStr">
-        <is>
-          <t>Con stock</t>
-        </is>
-      </c>
-      <c r="H47" s="8" t="n">
-        <v>5</v>
+      <c r="G47" s="15" t="inlineStr">
+        <is>
+          <t>Sin stock</t>
+        </is>
+      </c>
+      <c r="H47" s="15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="4" t="inlineStr">
-        <is>
-          <t>Manillares</t>
-        </is>
-      </c>
-      <c r="B48" s="4" t="inlineStr">
-        <is>
-          <t>Manillar Café Racer Universal 7/8 22mm Recto Negro</t>
-        </is>
-      </c>
-      <c r="C48" s="4" t="inlineStr">
-        <is>
-          <t>Café Racer</t>
-        </is>
-      </c>
-      <c r="D48" s="4" t="inlineStr">
-        <is>
-          <t>MAN-78-V3-NEG-001</t>
-        </is>
-      </c>
-      <c r="E48" s="5" t="n">
-        <v>890</v>
-      </c>
-      <c r="F48" s="6">
+      <c r="A48" s="12" t="inlineStr">
+        <is>
+          <t>Eléctrico</t>
+        </is>
+      </c>
+      <c r="B48" s="12" t="inlineStr">
+        <is>
+          <t>Señaleros LED Finos Universales 12V Para Moto - Amarillo</t>
+        </is>
+      </c>
+      <c r="C48" s="12" t="inlineStr">
+        <is>
+          <t>Señaleros LED</t>
+        </is>
+      </c>
+      <c r="D48" s="12" t="inlineStr">
+        <is>
+          <t>HP-Z0533</t>
+        </is>
+      </c>
+      <c r="E48" s="13" t="n">
+        <v>320</v>
+      </c>
+      <c r="F48" s="14">
         <f>ROUND(E48*0.9,0)</f>
         <v/>
       </c>
-      <c r="G48" s="7" t="inlineStr">
-        <is>
-          <t>Con stock</t>
-        </is>
-      </c>
-      <c r="H48" s="4" t="n">
-        <v>2</v>
+      <c r="G48" s="12" t="inlineStr">
+        <is>
+          <t>Sin stock</t>
+        </is>
+      </c>
+      <c r="H48" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="8" t="inlineStr">
-        <is>
-          <t>Protección</t>
-        </is>
-      </c>
-      <c r="B49" s="8" t="inlineStr">
-        <is>
-          <t>Guardamanos Protector Puños Moto Enduro Cross ABS - Negro</t>
-        </is>
-      </c>
-      <c r="C49" s="8" t="inlineStr">
-        <is>
-          <t>Guardamanos</t>
-        </is>
-      </c>
-      <c r="D49" s="8" t="inlineStr">
-        <is>
-          <t>HP-Q0211</t>
-        </is>
-      </c>
-      <c r="E49" s="9" t="n">
-        <v>690</v>
-      </c>
-      <c r="F49" s="10">
+      <c r="A49" s="15" t="inlineStr">
+        <is>
+          <t>Eléctrico</t>
+        </is>
+      </c>
+      <c r="B49" s="15" t="inlineStr">
+        <is>
+          <t>Señaleros Led Secuenciales Luz Amarilla Universales Moto Amarillo</t>
+        </is>
+      </c>
+      <c r="C49" s="15" t="inlineStr">
+        <is>
+          <t>Señaleros LED</t>
+        </is>
+      </c>
+      <c r="D49" s="15" t="inlineStr">
+        <is>
+          <t>SEÑAL01</t>
+        </is>
+      </c>
+      <c r="E49" s="16" t="n">
+        <v>350</v>
+      </c>
+      <c r="F49" s="17">
         <f>ROUND(E49*0.9,0)</f>
         <v/>
       </c>
-      <c r="G49" s="11" t="inlineStr">
-        <is>
-          <t>Con stock</t>
-        </is>
-      </c>
-      <c r="H49" s="8" t="n">
-        <v>5</v>
+      <c r="G49" s="15" t="inlineStr">
+        <is>
+          <t>Sin stock</t>
+        </is>
+      </c>
+      <c r="H49" s="15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="4" t="inlineStr">
-        <is>
-          <t>Protección</t>
-        </is>
-      </c>
-      <c r="B50" s="4" t="inlineStr">
-        <is>
-          <t>Guardamanos Protector Puños Moto Enduro Cross ABS - Azul</t>
-        </is>
-      </c>
-      <c r="C50" s="4" t="inlineStr">
-        <is>
-          <t>Guardamanos</t>
-        </is>
-      </c>
-      <c r="D50" s="4" t="inlineStr">
-        <is>
-          <t>HP-Q0212</t>
-        </is>
-      </c>
-      <c r="E50" s="5" t="n">
-        <v>690</v>
-      </c>
-      <c r="F50" s="6">
+      <c r="A50" s="12" t="inlineStr">
+        <is>
+          <t>Escapes</t>
+        </is>
+      </c>
+      <c r="B50" s="12" t="inlineStr">
+        <is>
+          <t>Escape SC Project 51mm Universal Moto - Negro</t>
+        </is>
+      </c>
+      <c r="C50" s="12" t="inlineStr">
+        <is>
+          <t>SC Project</t>
+        </is>
+      </c>
+      <c r="D50" s="12" t="inlineStr">
+        <is>
+          <t>HP-EXHAUST-GBLACK</t>
+        </is>
+      </c>
+      <c r="E50" s="13" t="n">
+        <v>2490</v>
+      </c>
+      <c r="F50" s="14">
         <f>ROUND(E50*0.9,0)</f>
         <v/>
       </c>
-      <c r="G50" s="7" t="inlineStr">
-        <is>
-          <t>Con stock</t>
-        </is>
-      </c>
-      <c r="H50" s="4" t="n">
-        <v>8</v>
+      <c r="G50" s="12" t="inlineStr">
+        <is>
+          <t>Sin stock</t>
+        </is>
+      </c>
+      <c r="H50" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="8" t="inlineStr">
-        <is>
-          <t>Protección</t>
-        </is>
-      </c>
-      <c r="B51" s="8" t="inlineStr">
-        <is>
-          <t>Guardamanos Protector Puños Moto Enduro Cross ABS - Rojo</t>
-        </is>
-      </c>
-      <c r="C51" s="8" t="inlineStr">
-        <is>
-          <t>Guardamanos</t>
-        </is>
-      </c>
-      <c r="D51" s="8" t="inlineStr">
-        <is>
-          <t>HP-Q0213</t>
-        </is>
-      </c>
-      <c r="E51" s="9" t="n">
-        <v>690</v>
-      </c>
-      <c r="F51" s="10">
+      <c r="A51" s="15" t="inlineStr">
+        <is>
+          <t>Escapes</t>
+        </is>
+      </c>
+      <c r="B51" s="15" t="inlineStr">
+        <is>
+          <t>Escape SC Project 51mm Universal Moto - Plateado</t>
+        </is>
+      </c>
+      <c r="C51" s="15" t="inlineStr">
+        <is>
+          <t>SC Project</t>
+        </is>
+      </c>
+      <c r="D51" s="15" t="inlineStr">
+        <is>
+          <t>HP-EXHAUST-GSILVER</t>
+        </is>
+      </c>
+      <c r="E51" s="16" t="n">
+        <v>2190</v>
+      </c>
+      <c r="F51" s="17">
         <f>ROUND(E51*0.9,0)</f>
         <v/>
       </c>
-      <c r="G51" s="11" t="inlineStr">
-        <is>
-          <t>Con stock</t>
-        </is>
-      </c>
-      <c r="H51" s="8" t="n">
-        <v>7</v>
+      <c r="G51" s="15" t="inlineStr">
+        <is>
+          <t>Sin stock</t>
+        </is>
+      </c>
+      <c r="H51" s="15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="4" t="inlineStr">
-        <is>
-          <t>Protección</t>
-        </is>
-      </c>
-      <c r="B52" s="4" t="inlineStr">
-        <is>
-          <t>Guardamanos Moto Con Señalero LED Integrado Negro</t>
-        </is>
-      </c>
-      <c r="C52" s="4" t="inlineStr">
-        <is>
-          <t>Guardamanos</t>
-        </is>
-      </c>
-      <c r="D52" s="4" t="inlineStr">
-        <is>
-          <t>HP-HS010</t>
-        </is>
-      </c>
-      <c r="E52" s="5" t="n">
-        <v>990</v>
-      </c>
-      <c r="F52" s="6">
+      <c r="A52" s="12" t="inlineStr">
+        <is>
+          <t>Escapes</t>
+        </is>
+      </c>
+      <c r="B52" s="12" t="inlineStr">
+        <is>
+          <t>Escape SC Project Boca Inclinada 51mm Negro Universal Moto</t>
+        </is>
+      </c>
+      <c r="C52" s="12" t="inlineStr">
+        <is>
+          <t>SC Project</t>
+        </is>
+      </c>
+      <c r="D52" s="12" t="inlineStr">
+        <is>
+          <t>AP-SLANTED01</t>
+        </is>
+      </c>
+      <c r="E52" s="13" t="n">
+        <v>2590</v>
+      </c>
+      <c r="F52" s="14">
         <f>ROUND(E52*0.9,0)</f>
         <v/>
       </c>
-      <c r="G52" s="7" t="inlineStr">
-        <is>
-          <t>Con stock</t>
-        </is>
-      </c>
-      <c r="H52" s="4" t="n">
-        <v>3</v>
+      <c r="G52" s="12" t="inlineStr">
+        <is>
+          <t>Sin stock</t>
+        </is>
+      </c>
+      <c r="H52" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="8" t="inlineStr">
-        <is>
-          <t>Protección</t>
-        </is>
-      </c>
-      <c r="B53" s="8" t="inlineStr">
-        <is>
-          <t>Protector De Levas Universal Moto ABS Varios Colores - Negro</t>
-        </is>
-      </c>
-      <c r="C53" s="8" t="inlineStr">
-        <is>
-          <t>Protectores de levas</t>
-        </is>
-      </c>
-      <c r="D53" s="8" t="inlineStr">
-        <is>
-          <t>HP-Q035B1</t>
-        </is>
-      </c>
-      <c r="E53" s="9" t="n">
-        <v>890</v>
-      </c>
-      <c r="F53" s="10">
+      <c r="A53" s="15" t="inlineStr">
+        <is>
+          <t>Escapes</t>
+        </is>
+      </c>
+      <c r="B53" s="15" t="inlineStr">
+        <is>
+          <t>Escape Tipo Akrapovic 51mm Universal Moto</t>
+        </is>
+      </c>
+      <c r="C53" s="15" t="inlineStr">
+        <is>
+          <t>Akrapovic</t>
+        </is>
+      </c>
+      <c r="D53" s="15" t="inlineStr">
+        <is>
+          <t>HP-EXHAUST-A</t>
+        </is>
+      </c>
+      <c r="E53" s="16" t="n">
+        <v>3990</v>
+      </c>
+      <c r="F53" s="17">
         <f>ROUND(E53*0.9,0)</f>
         <v/>
       </c>
-      <c r="G53" s="11" t="inlineStr">
-        <is>
-          <t>Con stock</t>
-        </is>
-      </c>
-      <c r="H53" s="8" t="n">
-        <v>10</v>
+      <c r="G53" s="15" t="inlineStr">
+        <is>
+          <t>Sin stock</t>
+        </is>
+      </c>
+      <c r="H53" s="15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="4" t="inlineStr">
-        <is>
-          <t>Protección</t>
-        </is>
-      </c>
-      <c r="B54" s="4" t="inlineStr">
-        <is>
-          <t>Protector De Levas Universal Moto ABS Varios Colores - Azul</t>
-        </is>
-      </c>
-      <c r="C54" s="4" t="inlineStr">
-        <is>
-          <t>Protectores de levas</t>
-        </is>
-      </c>
-      <c r="D54" s="4" t="inlineStr">
-        <is>
-          <t>HP-Q035B2</t>
-        </is>
-      </c>
-      <c r="E54" s="5" t="n">
-        <v>890</v>
-      </c>
-      <c r="F54" s="6">
+      <c r="A54" s="12" t="inlineStr">
+        <is>
+          <t>Escapes</t>
+        </is>
+      </c>
+      <c r="B54" s="12" t="inlineStr">
+        <is>
+          <t>Escape Yoshimura Fibra Carbono Universal Moto Deportivo 51mm</t>
+        </is>
+      </c>
+      <c r="C54" s="12" t="inlineStr">
+        <is>
+          <t>Yoshimura</t>
+        </is>
+      </c>
+      <c r="D54" s="12" t="inlineStr">
+        <is>
+          <t>AP-YOSHIMURA01</t>
+        </is>
+      </c>
+      <c r="E54" s="13" t="n">
+        <v>5890</v>
+      </c>
+      <c r="F54" s="14">
         <f>ROUND(E54*0.9,0)</f>
         <v/>
       </c>
-      <c r="G54" s="7" t="inlineStr">
-        <is>
-          <t>Con stock</t>
-        </is>
-      </c>
-      <c r="H54" s="4" t="n">
-        <v>2</v>
+      <c r="G54" s="12" t="inlineStr">
+        <is>
+          <t>Sin stock</t>
+        </is>
+      </c>
+      <c r="H54" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="15" t="inlineStr">
         <is>
-          <t>Protección</t>
+          <t>Baúles</t>
         </is>
       </c>
       <c r="B55" s="15" t="inlineStr">
         <is>
-          <t>Protector De Levas Universal Moto ABS Varios Colores - Rojo</t>
+          <t>Baúl Trasero Moto 28L ABS Clásico Seguro Universal Con Llave</t>
         </is>
       </c>
       <c r="C55" s="15" t="inlineStr">
         <is>
-          <t>Protectores de levas</t>
+          <t>Traseros</t>
         </is>
       </c>
       <c r="D55" s="15" t="inlineStr">
         <is>
-          <t>HP-Q035B3</t>
+          <t>AP-TAILBOXLED</t>
         </is>
       </c>
       <c r="E55" s="16" t="n">
-        <v>890</v>
+        <v>1750</v>
       </c>
       <c r="F55" s="17">
         <f>ROUND(E55*0.9,0)</f>
@@ -2407,636 +2407,44 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="4" t="inlineStr">
-        <is>
-          <t>Protección</t>
-        </is>
-      </c>
-      <c r="B56" s="4" t="inlineStr">
-        <is>
-          <t>Protector De Levas Freno Y Embrague Estilo Fibra De Carbono</t>
-        </is>
-      </c>
-      <c r="C56" s="4" t="inlineStr">
-        <is>
-          <t>Protectores de levas</t>
-        </is>
-      </c>
-      <c r="D56" s="4" t="inlineStr">
-        <is>
-          <t>HS-30006</t>
-        </is>
-      </c>
-      <c r="E56" s="5" t="n">
-        <v>690</v>
-      </c>
-      <c r="F56" s="6">
+      <c r="A56" s="12" t="inlineStr">
+        <is>
+          <t>Baúles</t>
+        </is>
+      </c>
+      <c r="B56" s="12" t="inlineStr">
+        <is>
+          <t>Baúl Trasero Moto 45L PP Alta Resistencia Universal Con Llave</t>
+        </is>
+      </c>
+      <c r="C56" s="12" t="inlineStr">
+        <is>
+          <t>Traseros</t>
+        </is>
+      </c>
+      <c r="D56" s="12" t="inlineStr">
+        <is>
+          <t>AP-TAILBOXSQ</t>
+        </is>
+      </c>
+      <c r="E56" s="13" t="n">
+        <v>3990</v>
+      </c>
+      <c r="F56" s="14">
         <f>ROUND(E56*0.9,0)</f>
         <v/>
       </c>
-      <c r="G56" s="7" t="inlineStr">
-        <is>
-          <t>Con stock</t>
-        </is>
-      </c>
-      <c r="H56" s="4" t="n">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="8" t="inlineStr">
-        <is>
-          <t>Protección</t>
-        </is>
-      </c>
-      <c r="B57" s="8" t="inlineStr">
-        <is>
-          <t>Protector De Levas Universal Aluminio Negro (uso deportivo)</t>
-        </is>
-      </c>
-      <c r="C57" s="8" t="inlineStr">
-        <is>
-          <t>Protectores de levas</t>
-        </is>
-      </c>
-      <c r="D57" s="8" t="inlineStr">
-        <is>
-          <t>MELI-MLU1039263040</t>
-        </is>
-      </c>
-      <c r="E57" s="9" t="n">
-        <v>690</v>
-      </c>
-      <c r="F57" s="10">
-        <f>ROUND(E57*0.9,0)</f>
-        <v/>
-      </c>
-      <c r="G57" s="11" t="inlineStr">
-        <is>
-          <t>Con stock</t>
-        </is>
-      </c>
-      <c r="H57" s="8" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="4" t="inlineStr">
-        <is>
-          <t>Protección</t>
-        </is>
-      </c>
-      <c r="B58" s="4" t="inlineStr">
-        <is>
-          <t>Slider Universal Aluminio Grande Moto Protector Anti Caídas</t>
-        </is>
-      </c>
-      <c r="C58" s="4" t="inlineStr">
-        <is>
-          <t>Sliders</t>
-        </is>
-      </c>
-      <c r="D58" s="4" t="inlineStr">
-        <is>
-          <t>FSB-002</t>
-        </is>
-      </c>
-      <c r="E58" s="5" t="n">
-        <v>1290</v>
-      </c>
-      <c r="F58" s="6">
-        <f>ROUND(E58*0.9,0)</f>
-        <v/>
-      </c>
-      <c r="G58" s="7" t="inlineStr">
-        <is>
-          <t>Con stock</t>
-        </is>
-      </c>
-      <c r="H58" s="4" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="8" t="inlineStr">
-        <is>
-          <t>Protección</t>
-        </is>
-      </c>
-      <c r="B59" s="8" t="inlineStr">
-        <is>
-          <t>Slider Universal Aluminio Moto Protector Anti Caídas Naranja</t>
-        </is>
-      </c>
-      <c r="C59" s="8" t="inlineStr">
-        <is>
-          <t>Sliders</t>
-        </is>
-      </c>
-      <c r="D59" s="8" t="inlineStr">
-        <is>
-          <t>FSB-003</t>
-        </is>
-      </c>
-      <c r="E59" s="9" t="n">
-        <v>1290</v>
-      </c>
-      <c r="F59" s="10">
-        <f>ROUND(E59*0.9,0)</f>
-        <v/>
-      </c>
-      <c r="G59" s="11" t="inlineStr">
-        <is>
-          <t>Con stock</t>
-        </is>
-      </c>
-      <c r="H59" s="8" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="4" t="inlineStr">
-        <is>
-          <t>Matrícula</t>
-        </is>
-      </c>
-      <c r="B60" s="4" t="inlineStr">
-        <is>
-          <t>Porta Matricula Rebatible Placa Patente Moto Rebatible</t>
-        </is>
-      </c>
-      <c r="C60" s="4" t="inlineStr">
-        <is>
-          <t>Rebatible</t>
-        </is>
-      </c>
-      <c r="D60" s="4" t="inlineStr">
-        <is>
-          <t>CPJ-62001</t>
-        </is>
-      </c>
-      <c r="E60" s="5" t="n">
-        <v>1290</v>
-      </c>
-      <c r="F60" s="6">
-        <f>ROUND(E60*0.9,0)</f>
-        <v/>
-      </c>
-      <c r="G60" s="7" t="inlineStr">
-        <is>
-          <t>Con stock</t>
-        </is>
-      </c>
-      <c r="H60" s="4" t="n">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="8" t="inlineStr">
-        <is>
-          <t>Matrícula</t>
-        </is>
-      </c>
-      <c r="B61" s="8" t="inlineStr">
-        <is>
-          <t>Porta Matricula Moto Rebatible Compacto Perfil Bajo</t>
-        </is>
-      </c>
-      <c r="C61" s="8" t="inlineStr">
-        <is>
-          <t>Rebatible</t>
-        </is>
-      </c>
-      <c r="D61" s="8" t="inlineStr">
-        <is>
-          <t>PATENTE1</t>
-        </is>
-      </c>
-      <c r="E61" s="9" t="n">
-        <v>890</v>
-      </c>
-      <c r="F61" s="10">
-        <f>ROUND(E61*0.9,0)</f>
-        <v/>
-      </c>
-      <c r="G61" s="11" t="inlineStr">
-        <is>
-          <t>Con stock</t>
-        </is>
-      </c>
-      <c r="H61" s="8" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="4" t="inlineStr">
-        <is>
-          <t>Carenado</t>
-        </is>
-      </c>
-      <c r="B62" s="4" t="inlineStr">
-        <is>
-          <t>Guardabarros Trasero Universal Moto ABS</t>
-        </is>
-      </c>
-      <c r="C62" s="4" t="inlineStr">
-        <is>
-          <t>Guardabarros</t>
-        </is>
-      </c>
-      <c r="D62" s="4" t="inlineStr">
-        <is>
-          <t>HP-DB004-B</t>
-        </is>
-      </c>
-      <c r="E62" s="5" t="n">
-        <v>1290</v>
-      </c>
-      <c r="F62" s="6">
-        <f>ROUND(E62*0.9,0)</f>
-        <v/>
-      </c>
-      <c r="G62" s="7" t="inlineStr">
-        <is>
-          <t>Con stock</t>
-        </is>
-      </c>
-      <c r="H62" s="4" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="15" t="inlineStr">
-        <is>
-          <t>Carenado</t>
-        </is>
-      </c>
-      <c r="B63" s="15" t="inlineStr">
-        <is>
-          <t>Deflector Parabrisas Para Moto Universal Transparente</t>
-        </is>
-      </c>
-      <c r="C63" s="15" t="inlineStr">
-        <is>
-          <t>Parabrisas</t>
-        </is>
-      </c>
-      <c r="D63" s="15" t="inlineStr">
-        <is>
-          <t>DFB-002</t>
-        </is>
-      </c>
-      <c r="E63" s="16" t="n">
-        <v>1750</v>
-      </c>
-      <c r="F63" s="17">
-        <f>ROUND(E63*0.9,0)</f>
-        <v/>
-      </c>
-      <c r="G63" s="15" t="inlineStr">
+      <c r="G56" s="12" t="inlineStr">
         <is>
           <t>Sin stock</t>
         </is>
       </c>
-      <c r="H63" s="15" t="n">
+      <c r="H56" s="12" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="12" t="inlineStr">
-        <is>
-          <t>Eléctrico</t>
-        </is>
-      </c>
-      <c r="B64" s="12" t="inlineStr">
-        <is>
-          <t>Señaleros LED Finos Universales 12V Para Moto - Amarillo</t>
-        </is>
-      </c>
-      <c r="C64" s="12" t="inlineStr">
-        <is>
-          <t>Señaleros LED</t>
-        </is>
-      </c>
-      <c r="D64" s="12" t="inlineStr">
-        <is>
-          <t>HP-Z0533</t>
-        </is>
-      </c>
-      <c r="E64" s="13" t="n">
-        <v>320</v>
-      </c>
-      <c r="F64" s="14">
-        <f>ROUND(E64*0.9,0)</f>
-        <v/>
-      </c>
-      <c r="G64" s="12" t="inlineStr">
-        <is>
-          <t>Sin stock</t>
-        </is>
-      </c>
-      <c r="H64" s="12" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="15" t="inlineStr">
-        <is>
-          <t>Eléctrico</t>
-        </is>
-      </c>
-      <c r="B65" s="15" t="inlineStr">
-        <is>
-          <t>Señaleros Led Secuenciales Luz Amarilla Universales Moto Amarillo</t>
-        </is>
-      </c>
-      <c r="C65" s="15" t="inlineStr">
-        <is>
-          <t>Señaleros LED</t>
-        </is>
-      </c>
-      <c r="D65" s="15" t="inlineStr">
-        <is>
-          <t>SEÑAL01</t>
-        </is>
-      </c>
-      <c r="E65" s="16" t="n">
-        <v>350</v>
-      </c>
-      <c r="F65" s="17">
-        <f>ROUND(E65*0.9,0)</f>
-        <v/>
-      </c>
-      <c r="G65" s="15" t="inlineStr">
-        <is>
-          <t>Sin stock</t>
-        </is>
-      </c>
-      <c r="H65" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="12" t="inlineStr">
-        <is>
-          <t>Escapes</t>
-        </is>
-      </c>
-      <c r="B66" s="12" t="inlineStr">
-        <is>
-          <t>Escape SC Project 51mm Universal Moto - Negro</t>
-        </is>
-      </c>
-      <c r="C66" s="12" t="inlineStr">
-        <is>
-          <t>SC Project</t>
-        </is>
-      </c>
-      <c r="D66" s="12" t="inlineStr">
-        <is>
-          <t>HP-EXHAUST-GBLACK</t>
-        </is>
-      </c>
-      <c r="E66" s="13" t="n">
-        <v>2490</v>
-      </c>
-      <c r="F66" s="14">
-        <f>ROUND(E66*0.9,0)</f>
-        <v/>
-      </c>
-      <c r="G66" s="12" t="inlineStr">
-        <is>
-          <t>Sin stock</t>
-        </is>
-      </c>
-      <c r="H66" s="12" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="15" t="inlineStr">
-        <is>
-          <t>Escapes</t>
-        </is>
-      </c>
-      <c r="B67" s="15" t="inlineStr">
-        <is>
-          <t>Escape SC Project 51mm Universal Moto - Plateado</t>
-        </is>
-      </c>
-      <c r="C67" s="15" t="inlineStr">
-        <is>
-          <t>SC Project</t>
-        </is>
-      </c>
-      <c r="D67" s="15" t="inlineStr">
-        <is>
-          <t>HP-EXHAUST-GSILVER</t>
-        </is>
-      </c>
-      <c r="E67" s="16" t="n">
-        <v>2190</v>
-      </c>
-      <c r="F67" s="17">
-        <f>ROUND(E67*0.9,0)</f>
-        <v/>
-      </c>
-      <c r="G67" s="15" t="inlineStr">
-        <is>
-          <t>Sin stock</t>
-        </is>
-      </c>
-      <c r="H67" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="12" t="inlineStr">
-        <is>
-          <t>Escapes</t>
-        </is>
-      </c>
-      <c r="B68" s="12" t="inlineStr">
-        <is>
-          <t>Escape SC Project Boca Inclinada 51mm Negro Universal Moto</t>
-        </is>
-      </c>
-      <c r="C68" s="12" t="inlineStr">
-        <is>
-          <t>SC Project</t>
-        </is>
-      </c>
-      <c r="D68" s="12" t="inlineStr">
-        <is>
-          <t>AP-SLANTED01</t>
-        </is>
-      </c>
-      <c r="E68" s="13" t="n">
-        <v>2590</v>
-      </c>
-      <c r="F68" s="14">
-        <f>ROUND(E68*0.9,0)</f>
-        <v/>
-      </c>
-      <c r="G68" s="12" t="inlineStr">
-        <is>
-          <t>Sin stock</t>
-        </is>
-      </c>
-      <c r="H68" s="12" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="15" t="inlineStr">
-        <is>
-          <t>Escapes</t>
-        </is>
-      </c>
-      <c r="B69" s="15" t="inlineStr">
-        <is>
-          <t>Escape Tipo Akrapovic 51mm Universal Moto</t>
-        </is>
-      </c>
-      <c r="C69" s="15" t="inlineStr">
-        <is>
-          <t>Akrapovic</t>
-        </is>
-      </c>
-      <c r="D69" s="15" t="inlineStr">
-        <is>
-          <t>HP-EXHAUST-A</t>
-        </is>
-      </c>
-      <c r="E69" s="16" t="n">
-        <v>3990</v>
-      </c>
-      <c r="F69" s="17">
-        <f>ROUND(E69*0.9,0)</f>
-        <v/>
-      </c>
-      <c r="G69" s="15" t="inlineStr">
-        <is>
-          <t>Sin stock</t>
-        </is>
-      </c>
-      <c r="H69" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="12" t="inlineStr">
-        <is>
-          <t>Escapes</t>
-        </is>
-      </c>
-      <c r="B70" s="12" t="inlineStr">
-        <is>
-          <t>Escape Yoshimura Fibra Carbono Universal Moto Deportivo 51mm</t>
-        </is>
-      </c>
-      <c r="C70" s="12" t="inlineStr">
-        <is>
-          <t>Yoshimura</t>
-        </is>
-      </c>
-      <c r="D70" s="12" t="inlineStr">
-        <is>
-          <t>AP-YOSHIMURA01</t>
-        </is>
-      </c>
-      <c r="E70" s="13" t="n">
-        <v>5890</v>
-      </c>
-      <c r="F70" s="14">
-        <f>ROUND(E70*0.9,0)</f>
-        <v/>
-      </c>
-      <c r="G70" s="12" t="inlineStr">
-        <is>
-          <t>Sin stock</t>
-        </is>
-      </c>
-      <c r="H70" s="12" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="15" t="inlineStr">
-        <is>
-          <t>Baúles</t>
-        </is>
-      </c>
-      <c r="B71" s="15" t="inlineStr">
-        <is>
-          <t>Baúl Trasero Moto 28L ABS Clásico Seguro Universal Con Llave</t>
-        </is>
-      </c>
-      <c r="C71" s="15" t="inlineStr">
-        <is>
-          <t>Traseros</t>
-        </is>
-      </c>
-      <c r="D71" s="15" t="inlineStr">
-        <is>
-          <t>AP-TAILBOXLED</t>
-        </is>
-      </c>
-      <c r="E71" s="16" t="n">
-        <v>1750</v>
-      </c>
-      <c r="F71" s="17">
-        <f>ROUND(E71*0.9,0)</f>
-        <v/>
-      </c>
-      <c r="G71" s="15" t="inlineStr">
-        <is>
-          <t>Sin stock</t>
-        </is>
-      </c>
-      <c r="H71" s="15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="12" t="inlineStr">
-        <is>
-          <t>Baúles</t>
-        </is>
-      </c>
-      <c r="B72" s="12" t="inlineStr">
-        <is>
-          <t>Baúl Trasero Moto 45L PP Alta Resistencia Universal Con Llave</t>
-        </is>
-      </c>
-      <c r="C72" s="12" t="inlineStr">
-        <is>
-          <t>Traseros</t>
-        </is>
-      </c>
-      <c r="D72" s="12" t="inlineStr">
-        <is>
-          <t>AP-TAILBOXSQ</t>
-        </is>
-      </c>
-      <c r="E72" s="13" t="n">
-        <v>3990</v>
-      </c>
-      <c r="F72" s="14">
-        <f>ROUND(E72*0.9,0)</f>
-        <v/>
-      </c>
-      <c r="G72" s="12" t="inlineStr">
-        <is>
-          <t>Sin stock</t>
-        </is>
-      </c>
-      <c r="H72" s="12" t="n">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A5:H72"/>
+  <autoFilter ref="A5:H56"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>